<commit_message>
docs(testing): add E10-S02 cases for Technical Support reconfirmation (SCRUM-244)
TC_E10S02_05, _06 and _08 now expect staffed Technical Support requests to be
flagged and their technicians told (T-103); TC_E10S02_10 to _13 add the
non-overlapping Session change, readiness, reconfirmation at the shifted time
and the busy-technician refusal. TC_E10S02_05 loses a leftover second block
that filled its exported row. Workbook re-exported; tc-coverage regenerated.
</commit_message>
<xml_diff>
--- a/docs/testing/PROJECT TEST CASES CAA 311026.xlsx
+++ b/docs/testing/PROJECT TEST CASES CAA 311026.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J380"/>
+  <dimension ref="A1:J384"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -17751,24 +17751,23 @@
       </c>
       <c r="G331" s="2" t="inlineStr">
         <is>
-          <t>A event of "Tech Conference 2026" has a confirmed venue and reserved equipment</t>
+          <t>Event E-1 has two Sessions; each has a confirmed venue booking and equipment reservation; a staffed Technical Support request covers Session A's time</t>
         </is>
       </c>
       <c r="H331" s="2" t="inlineStr">
         <is>
-          <t>1. Log in as coordinator_1@connectsphere.com
-  2. Change the event's date from 15/11/2026 to 20/11/2026
-  3. Save</t>
+          <t>1. Change Session A date/time
+2. Review Session A and B arrangements</t>
         </is>
       </c>
       <c r="I331" s="2" t="inlineStr">
         <is>
-          <t>Date: 15/11/2026 -&gt; 20/11/2026</t>
+          <t>Only Session A changes from 2027-03-12 09:00–11:00 to 2027-03-13 09:00–11:00 | Support request: 2027-03-12 08:00–11:00, one technician assigned</t>
         </is>
       </c>
       <c r="J331" s="2" t="inlineStr">
         <is>
-          <t>Both the venue booking and the equipment reservations for this event are flagged as requiring reconfirmation</t>
+          <t>Session A booking and equipment reservation, and the staffed Technical Support request overlapping Session A's previous time, are flagged; Session B arrangements remain confirmed and unchanged</t>
         </is>
       </c>
     </row>
@@ -17783,7 +17782,7 @@
       </c>
       <c r="C332" s="2" t="inlineStr">
         <is>
-          <t>E10-S02 (checklist: Venue Staff and Technical Support Staff both notified)</t>
+          <t>E10-S02 - Scenario 6 (Affected staff notified); T-103</t>
         </is>
       </c>
       <c r="D332" s="2" t="inlineStr">
@@ -17821,7 +17820,7 @@
       </c>
       <c r="J332" s="2" t="inlineStr">
         <is>
-          <t>Both venue_staff_1@connectsphere.com and tech_support_1@connectsphere.com receive a notification about the change requiring reconfirmation</t>
+          <t>Both venue_staff_1@connectsphere.com and tech_support_1@connectsphere.com receive a notification about the change requiring reconfirmation; tech_support_1's notification covers the flagged Technical Support request as well as the equipment</t>
         </is>
       </c>
     </row>
@@ -17888,7 +17887,7 @@
       </c>
       <c r="C334" s="2" t="inlineStr">
         <is>
-          <t>E10-S02 - Scenario 5 (Session date/time change flags its arrangements); T-79</t>
+          <t>E10-S02 - Scenario 5 (Session date/time change flags its arrangements); T-79; T-103</t>
         </is>
       </c>
       <c r="D334" s="2" t="inlineStr">
@@ -17908,7 +17907,7 @@
       </c>
       <c r="G334" s="2" t="inlineStr">
         <is>
-          <t>Event E-1 has two Sessions with confirmed venue bookings and equipment reservations</t>
+          <t>Event E-1 has two Sessions with confirmed venue bookings and equipment reservations, and two staffed Technical Support requests</t>
         </is>
       </c>
       <c r="H334" s="2" t="inlineStr">
@@ -17924,7 +17923,7 @@
       </c>
       <c r="J334" s="2" t="inlineStr">
         <is>
-          <t>Both Sessions’ venue bookings and equipment reservations are flagged for reconfirmation</t>
+          <t>Both Sessions’ venue bookings and equipment reservations, and both staffed Technical Support requests, are flagged for reconfirmation</t>
         </is>
       </c>
     </row>
@@ -17981,252 +17980,458 @@
       </c>
     </row>
     <row r="336">
-      <c r="A336" s="2" t="inlineStr">
+      <c r="A336" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B336" s="2" t="inlineStr">
+        <is>
+          <t>E10-S02</t>
+        </is>
+      </c>
+      <c r="C336" s="2" t="inlineStr">
+        <is>
+          <t>E10-S02 - Scenario 5 (Session date/time change flags its arrangements); T-103</t>
+        </is>
+      </c>
+      <c r="D336" s="2" t="inlineStr">
+        <is>
+          <t>4 - Negative</t>
+        </is>
+      </c>
+      <c r="E336" s="2" t="inlineStr">
+        <is>
+          <t>TC_E10S02_10</t>
+        </is>
+      </c>
+      <c r="F336" s="2" t="inlineStr">
+        <is>
+          <t>A Session change should not flag a Technical Support request that does not overlap that Session</t>
+        </is>
+      </c>
+      <c r="G336" s="2" t="inlineStr">
+        <is>
+          <t>Event E-1 has two Sessions; a staffed Technical Support request covers only Session B's time</t>
+        </is>
+      </c>
+      <c r="H336" s="2" t="inlineStr">
+        <is>
+          <t>1. Change Session A date/time
+2. Review the Technical Support request</t>
+        </is>
+      </c>
+      <c r="I336" s="2" t="inlineStr">
+        <is>
+          <t>Session A: 2027-03-12 09:00–11:00 -&gt; 2027-03-13 09:00–11:00 | Support request: 2027-03-12 14:00–17:00 (Session B)</t>
+        </is>
+      </c>
+      <c r="J336" s="2" t="inlineStr">
+        <is>
+          <t>The Technical Support request is not flagged and keeps its time; its technician is not notified</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B337" s="2" t="inlineStr">
+        <is>
+          <t>E10-S02</t>
+        </is>
+      </c>
+      <c r="C337" s="2" t="inlineStr">
+        <is>
+          <t>E10-S02 - Scenario 5 (flagged support is outstanding); T-103; E08-S04 Scenario 4</t>
+        </is>
+      </c>
+      <c r="D337" s="2" t="inlineStr">
+        <is>
+          <t>3 - Integration / regression</t>
+        </is>
+      </c>
+      <c r="E337" s="2" t="inlineStr">
+        <is>
+          <t>TC_E10S02_11</t>
+        </is>
+      </c>
+      <c r="F337" s="2" t="inlineStr">
+        <is>
+          <t>A flagged Technical Support request should keep a reverted Event out of Safety Review</t>
+        </is>
+      </c>
+      <c r="G337" s="2" t="inlineStr">
+        <is>
+          <t>Event "Charity Run" was Confirmed, then reverted to Planning; a date change flagged its venue booking, equipment reservation and staffed Technical Support request</t>
+        </is>
+      </c>
+      <c r="H337" s="2" t="inlineStr">
+        <is>
+          <t>1. Venue Staff reconfirm the booking
+2. Technical Support Staff re-save the equipment reservation
+3. Open the Event's readiness page</t>
+        </is>
+      </c>
+      <c r="I337" s="2" t="inlineStr">
+        <is>
+          <t>Technical Support request still flagged</t>
+        </is>
+      </c>
+      <c r="J337" s="2" t="inlineStr">
+        <is>
+          <t>The Event stays in Planning; the readiness page lists the Technical Support request as outstanding; no Safety Review notification is sent</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B338" s="2" t="inlineStr">
+        <is>
+          <t>E10-S02</t>
+        </is>
+      </c>
+      <c r="C338" s="2" t="inlineStr">
+        <is>
+          <t>E10-S02 - Scenario 5 (reconfirmed at the new time); T-103</t>
+        </is>
+      </c>
+      <c r="D338" s="2" t="inlineStr">
+        <is>
+          <t>2 - Happy Path</t>
+        </is>
+      </c>
+      <c r="E338" s="2" t="inlineStr">
+        <is>
+          <t>TC_E10S02_12</t>
+        </is>
+      </c>
+      <c r="F338" s="2" t="inlineStr">
+        <is>
+          <t>Reconfirming a flagged Technical Support request should move it and its technicians to the new time</t>
+        </is>
+      </c>
+      <c r="G338" s="2" t="inlineStr">
+        <is>
+          <t>Event "Charity Run" moved from 5 Dec 2026 07:00–12:00 to 12 Dec 2026 07:00–12:00; its staffed Technical Support request (5 Dec 06:00–12:00, tech_support_1 assigned) is flagged; every other arrangement is already reconfirmed; the Event was Confirmed before</t>
+        </is>
+      </c>
+      <c r="H338" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in as tech_support_1@connectsphere.com
+2. Open the Technical Support requests to reconfirm
+3. Reconfirm the Charity Run request</t>
+        </is>
+      </c>
+      <c r="I338" s="2" t="inlineStr">
+        <is>
+          <t>Shift: +7 days, same length</t>
+        </is>
+      </c>
+      <c r="J338" s="2" t="inlineStr">
+        <is>
+          <t>The request and tech_support_1's assignment move to 12 Dec 2026 06:00–12:00; the flag clears; the reconfirmation is in the Activity log; the Coordinator is notified; because it was the last outstanding arrangement, the Event enters Safety Review and the Safety Officer is notified</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B339" s="2" t="inlineStr">
+        <is>
+          <t>E10-S02</t>
+        </is>
+      </c>
+      <c r="C339" s="2" t="inlineStr">
+        <is>
+          <t>E10-S02 - Scenario 5 (reconfirmed at the new time); T-103</t>
+        </is>
+      </c>
+      <c r="D339" s="2" t="inlineStr">
+        <is>
+          <t>4 - Negative</t>
+        </is>
+      </c>
+      <c r="E339" s="2" t="inlineStr">
+        <is>
+          <t>TC_E10S02_13</t>
+        </is>
+      </c>
+      <c r="F339" s="2" t="inlineStr">
+        <is>
+          <t>Reconfirming a Technical Support request should be refused when an assigned technician is busy at the new time</t>
+        </is>
+      </c>
+      <c r="G339" s="2" t="inlineStr">
+        <is>
+          <t>A flagged Technical Support request moves to 12 Dec 2026 06:00–12:00; its technician tech_support_1 is already assigned to another event on 12 Dec 2026 10:00–14:00</t>
+        </is>
+      </c>
+      <c r="H339" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in as a Technical Support Staff member
+2. Reconfirm the flagged request</t>
+        </is>
+      </c>
+      <c r="I339" s="2" t="inlineStr">
+        <is>
+          <t>Overlap: 12 Dec 2026 10:00–12:00</t>
+        </is>
+      </c>
+      <c r="J339" s="2" t="inlineStr">
+        <is>
+          <t>The reconfirmation is refused with a message naming the busy technician and the overlapping time; the request stays flagged at its old time and nothing else changes</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" s="2" t="inlineStr">
         <is>
           <t>Unassigned</t>
         </is>
       </c>
-      <c r="B336" s="2" t="inlineStr">
+      <c r="B340" s="2" t="inlineStr">
         <is>
           <t>E10-S03</t>
         </is>
       </c>
-      <c r="C336" s="2" t="inlineStr">
+      <c r="C340" s="2" t="inlineStr">
         <is>
           <t>E10-S03 - Scenario 1 (Session date change flags its arrangements)</t>
         </is>
       </c>
-      <c r="D336" s="2" t="inlineStr">
+      <c r="D340" s="2" t="inlineStr">
         <is>
           <t>3 - Integration / regression</t>
         </is>
       </c>
-      <c r="E336" s="2" t="inlineStr">
+      <c r="E340" s="2" t="inlineStr">
         <is>
           <t>TC_E10S03_01</t>
         </is>
       </c>
-      <c r="F336" s="2" t="inlineStr">
+      <c r="F340" s="2" t="inlineStr">
         <is>
           <t>Changing one Session date should flag only that Session’s arrangements</t>
         </is>
       </c>
-      <c r="G336" s="2" t="inlineStr">
+      <c r="G340" s="2" t="inlineStr">
         <is>
           <t>Event E-1 has two Sessions, each with confirmed venue and equipment arrangements</t>
         </is>
       </c>
-      <c r="H336" s="2" t="inlineStr">
+      <c r="H340" s="2" t="inlineStr">
         <is>
           <t>1. Change Session A date/time
 2. Review all arrangements</t>
         </is>
       </c>
-      <c r="I336" s="2" t="inlineStr">
+      <c r="I340" s="2" t="inlineStr">
         <is>
           <t>Session A and B have distinct bookings</t>
         </is>
       </c>
-      <c r="J336" s="2" t="inlineStr">
+      <c r="J340" s="2" t="inlineStr">
         <is>
           <t>Only Session A’s arrangements are flagged; none are silently moved</t>
         </is>
       </c>
     </row>
-    <row r="337">
-      <c r="A337" s="2" t="inlineStr">
+    <row r="341">
+      <c r="A341" s="2" t="inlineStr">
         <is>
           <t>Unassigned</t>
         </is>
       </c>
-      <c r="B337" s="2" t="inlineStr">
+      <c r="B341" s="2" t="inlineStr">
         <is>
           <t>E10-S03</t>
         </is>
       </c>
-      <c r="C337" s="2" t="inlineStr">
+      <c r="C341" s="2" t="inlineStr">
         <is>
           <t>E10-S03 - Scenario 2 (Event-wide date change flags all Sessions)</t>
         </is>
       </c>
-      <c r="D337" s="2" t="inlineStr">
+      <c r="D341" s="2" t="inlineStr">
         <is>
           <t>3 - Integration / regression</t>
         </is>
       </c>
-      <c r="E337" s="2" t="inlineStr">
+      <c r="E341" s="2" t="inlineStr">
         <is>
           <t>TC_E10S03_02</t>
         </is>
       </c>
-      <c r="F337" s="2" t="inlineStr">
+      <c r="F341" s="2" t="inlineStr">
         <is>
           <t>An Event-wide reschedule should flag arrangements for every Session</t>
         </is>
       </c>
-      <c r="G337" s="2" t="inlineStr">
+      <c r="G341" s="2" t="inlineStr">
         <is>
           <t>Event E-1 has multiple Sessions with confirmed arrangements</t>
         </is>
       </c>
-      <c r="H337" s="2" t="inlineStr">
+      <c r="H341" s="2" t="inlineStr">
         <is>
           <t>1. Change the Event-wide date
 2. Review all Session arrangements</t>
         </is>
       </c>
-      <c r="I337" s="2" t="inlineStr">
+      <c r="I341" s="2" t="inlineStr">
         <is>
           <t>Event E-1: two Sessions</t>
         </is>
       </c>
-      <c r="J337" s="2" t="inlineStr">
+      <c r="J341" s="2" t="inlineStr">
         <is>
           <t>Every Session booking and equipment reservation is flagged for reconfirmation</t>
         </is>
       </c>
     </row>
-    <row r="338">
-      <c r="A338" s="2" t="inlineStr">
+    <row r="342">
+      <c r="A342" s="2" t="inlineStr">
         <is>
           <t>Unassigned</t>
         </is>
       </c>
-      <c r="B338" s="2" t="inlineStr">
+      <c r="B342" s="2" t="inlineStr">
         <is>
           <t>E10-S03</t>
         </is>
       </c>
-      <c r="C338" s="2" t="inlineStr">
+      <c r="C342" s="2" t="inlineStr">
         <is>
           <t>E10-S03 - Scenario 3 (Registered Attendees notified)</t>
         </is>
       </c>
-      <c r="D338" s="2" t="inlineStr">
+      <c r="D342" s="2" t="inlineStr">
         <is>
           <t>3 - Cross-cutting (notification consistency)</t>
         </is>
       </c>
-      <c r="E338" s="2" t="inlineStr">
+      <c r="E342" s="2" t="inlineStr">
         <is>
           <t>TC_E10S03_03</t>
         </is>
       </c>
-      <c r="F338" s="2" t="inlineStr">
+      <c r="F342" s="2" t="inlineStr">
         <is>
           <t>Registered Attendees should be notified of the new Event and Session dates</t>
         </is>
       </c>
-      <c r="G338" s="2" t="inlineStr">
+      <c r="G342" s="2" t="inlineStr">
         <is>
           <t>Attendees are registered for Event E-1 and selected different Sessions</t>
         </is>
       </c>
-      <c r="H338" s="2" t="inlineStr">
+      <c r="H342" s="2" t="inlineStr">
         <is>
           <t>1. Reschedule the Event and one Session
 2. Check the registered attendees’ notifications</t>
         </is>
       </c>
-      <c r="I338" s="2" t="inlineStr">
+      <c r="I342" s="2" t="inlineStr">
         <is>
           <t>New Event and Session dates are recorded</t>
         </is>
       </c>
-      <c r="J338" s="2" t="inlineStr">
+      <c r="J342" s="2" t="inlineStr">
         <is>
           <t>All registered Attendees are notified of the new Event and Session dates/times</t>
         </is>
       </c>
     </row>
-    <row r="339">
-      <c r="A339" s="2" t="inlineStr">
+    <row r="343">
+      <c r="A343" s="2" t="inlineStr">
         <is>
           <t>Unassigned</t>
         </is>
       </c>
-      <c r="B339" s="2" t="inlineStr">
+      <c r="B343" s="2" t="inlineStr">
         <is>
           <t>E10-S03</t>
         </is>
       </c>
-      <c r="C339" s="2" t="inlineStr">
+      <c r="C343" s="2" t="inlineStr">
         <is>
           <t>E10-S03 - Scenario 4 (Pending change requests closed on terminal Event); C-77/T-88</t>
         </is>
       </c>
-      <c r="D339" s="2" t="inlineStr">
+      <c r="D343" s="2" t="inlineStr">
         <is>
           <t>3 - Integration / regression</t>
         </is>
       </c>
-      <c r="E339" s="2" t="inlineStr">
+      <c r="E343" s="2" t="inlineStr">
         <is>
           <t>TC_E10S03_04</t>
         </is>
       </c>
-      <c r="F339" s="2" t="inlineStr">
+      <c r="F343" s="2" t="inlineStr">
         <is>
           <t>Pending change requests should become Obsolete when a rescheduled Event later becomes terminal</t>
         </is>
       </c>
-      <c r="G339" s="2" t="inlineStr">
+      <c r="G343" s="2" t="inlineStr">
         <is>
           <t>Event E-1 has a Pending change request while a reschedule is in progress</t>
         </is>
       </c>
-      <c r="H339" s="2" t="inlineStr">
+      <c r="H343" s="2" t="inlineStr">
         <is>
           <t>1. Complete or cancel Event E-1
 2. Inspect the other Pending change request and its history</t>
         </is>
       </c>
-      <c r="I339" s="2" t="inlineStr">
+      <c r="I343" s="2" t="inlineStr">
         <is>
           <t>Event E-1: terminal status</t>
         </is>
       </c>
-      <c r="J339" s="2" t="inlineStr">
+      <c r="J343" s="2" t="inlineStr">
         <is>
           <t>The remaining Pending request becomes Obsolete and the transition is recorded in history</t>
         </is>
       </c>
     </row>
-    <row r="340">
-      <c r="A340" s="2" t="n">
+    <row r="344">
+      <c r="A344" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="B340" s="2" t="inlineStr">
+      <c r="B344" s="2" t="inlineStr">
         <is>
           <t>E10-S04</t>
         </is>
       </c>
-      <c r="C340" s="2" t="inlineStr">
+      <c r="C344" s="2" t="inlineStr">
         <is>
           <t>E10-S04 - Scenario 1 (Event cancelled and Session arrangements released); T-79</t>
         </is>
       </c>
-      <c r="D340" s="2" t="inlineStr">
+      <c r="D344" s="2" t="inlineStr">
         <is>
           <t>3 - Integration / regression</t>
         </is>
       </c>
-      <c r="E340" s="2" t="inlineStr">
+      <c r="E344" s="2" t="inlineStr">
         <is>
           <t>TC_E10S04_01</t>
         </is>
       </c>
-      <c r="F340" s="2" t="inlineStr">
+      <c r="F344" s="2" t="inlineStr">
         <is>
           <t>Cancelling an Event should release all Session bookings and equipment reservations</t>
         </is>
       </c>
-      <c r="G340" s="2" t="inlineStr">
+      <c r="G344" s="2" t="inlineStr">
         <is>
           <t>Event "Product Launch Night" has status "Confirmed" with a confirmed venue "Small Room" and reserved equipment</t>
         </is>
       </c>
-      <c r="H340" s="2" t="inlineStr">
+      <c r="H344" s="2" t="inlineStr">
         <is>
           <t>1. Log in as coordinator_1@connectsphere.com
   2. Open event "Product Launch Night"
@@ -18235,156 +18440,156 @@
   5. Confirm</t>
         </is>
       </c>
-      <c r="I340" s="2" t="inlineStr">
+      <c r="I344" s="2" t="inlineStr">
         <is>
           <t>Cancellation reason: "Insufficient sponsor funding"</t>
         </is>
       </c>
-      <c r="J340" s="2" t="inlineStr">
+      <c r="J344" s="2" t="inlineStr">
         <is>
           <t>The status becomes "Cancelled"; "Small Room"'s booking and the reserved equipment are released, the venue calendar is updated, and affected staff are notified</t>
         </is>
       </c>
     </row>
-    <row r="341">
-      <c r="A341" s="2" t="n">
+    <row r="345">
+      <c r="A345" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="B341" s="2" t="inlineStr">
+      <c r="B345" s="2" t="inlineStr">
         <is>
           <t>E10-S04</t>
         </is>
       </c>
-      <c r="C341" s="2" t="inlineStr">
+      <c r="C345" s="2" t="inlineStr">
         <is>
           <t>E10-S04 - Scenario 2 (Attendees and waitlist notified)</t>
         </is>
       </c>
-      <c r="D341" s="2" t="inlineStr">
+      <c r="D345" s="2" t="inlineStr">
         <is>
           <t>2 - Happy Path</t>
         </is>
       </c>
-      <c r="E341" s="2" t="inlineStr">
+      <c r="E345" s="2" t="inlineStr">
         <is>
           <t>TC_E10S04_03</t>
         </is>
       </c>
-      <c r="F341" s="2" t="inlineStr">
+      <c r="F345" s="2" t="inlineStr">
         <is>
           <t>Verify that cancelling a event should notify all of its registered and waitlisted Attendees</t>
         </is>
       </c>
-      <c r="G341" s="2" t="inlineStr">
+      <c r="G345" s="2" t="inlineStr">
         <is>
           <t>The event of "Tech Conference 2026" being cancelled has attendee_a@example.com registered and attendee_l@example.com waitlisted</t>
         </is>
       </c>
-      <c r="H341" s="2" t="inlineStr">
+      <c r="H345" s="2" t="inlineStr">
         <is>
           <t>1. Log in as coordinator_1@connectsphere.com
   2. Cancel the event
   3. Check notifications for attendee_a@example.com and attendee_l@example.com</t>
         </is>
       </c>
-      <c r="I341" s="2" t="inlineStr">
+      <c r="I345" s="2" t="inlineStr">
         <is>
           <t>Registered: attendee_a@example.com | Waitlisted: attendee_l@example.com</t>
         </is>
       </c>
-      <c r="J341" s="2" t="inlineStr">
+      <c r="J345" s="2" t="inlineStr">
         <is>
           <t>Both attendee_a@example.com and attendee_l@example.com receive a notification of the cancellation</t>
         </is>
       </c>
     </row>
-    <row r="342">
-      <c r="A342" s="2" t="n">
+    <row r="346">
+      <c r="A346" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="B342" s="2" t="inlineStr">
+      <c r="B346" s="2" t="inlineStr">
         <is>
           <t>E10-S04</t>
         </is>
       </c>
-      <c r="C342" s="2" t="inlineStr">
+      <c r="C346" s="2" t="inlineStr">
         <is>
           <t>E10-S04 - Scenario 3 (Cancelled event read-only)</t>
         </is>
       </c>
-      <c r="D342" s="2" t="inlineStr">
+      <c r="D346" s="2" t="inlineStr">
         <is>
           <t>2 - Happy Path</t>
         </is>
       </c>
-      <c r="E342" s="2" t="inlineStr">
+      <c r="E346" s="2" t="inlineStr">
         <is>
           <t>TC_E10S04_04</t>
         </is>
       </c>
-      <c r="F342" s="2" t="inlineStr">
+      <c r="F346" s="2" t="inlineStr">
         <is>
           <t>Verify that a cancelled event should be read-only and show its cancellation reason and date to any viewer</t>
         </is>
       </c>
-      <c r="G342" s="2" t="inlineStr">
+      <c r="G346" s="2" t="inlineStr">
         <is>
           <t>Event "Product Launch Night" was cancelled on 12/09/2026 with reason "Insufficient sponsor funding" (per TC_E10S04_01)</t>
         </is>
       </c>
-      <c r="H342" s="2" t="inlineStr">
+      <c r="H346" s="2" t="inlineStr">
         <is>
           <t>1. Log in as any user with access (e.g. organiser_a@clienta.com)
   2. Open the cancelled event "Product Launch Night"
   3. Attempt to edit any field</t>
         </is>
       </c>
-      <c r="I342" s="2" t="inlineStr">
+      <c r="I346" s="2" t="inlineStr">
         <is>
           <t>Cancellation reason: "Insufficient sponsor funding" | Date: 12/09/2026</t>
         </is>
       </c>
-      <c r="J342" s="2" t="inlineStr">
+      <c r="J346" s="2" t="inlineStr">
         <is>
           <t>The event shows "Cancelled on 12 September 2026 - Insufficient sponsor funding"; all fields are read-only</t>
         </is>
       </c>
     </row>
-    <row r="343">
-      <c r="A343" s="2" t="n">
+    <row r="347">
+      <c r="A347" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="B343" s="2" t="inlineStr">
+      <c r="B347" s="2" t="inlineStr">
         <is>
           <t>E10-S04</t>
         </is>
       </c>
-      <c r="C343" s="2" t="inlineStr">
+      <c r="C347" s="2" t="inlineStr">
         <is>
           <t>E10-S04 - Scenario 4 (Organiser cancellation becomes a request)</t>
         </is>
       </c>
-      <c r="D343" s="2" t="inlineStr">
+      <c r="D347" s="2" t="inlineStr">
         <is>
           <t>4 - Negative</t>
         </is>
       </c>
-      <c r="E343" s="2" t="inlineStr">
+      <c r="E347" s="2" t="inlineStr">
         <is>
           <t>TC_E10S04_05</t>
         </is>
       </c>
-      <c r="F343" s="2" t="inlineStr">
+      <c r="F347" s="2" t="inlineStr">
         <is>
           <t>Verify that an Event Organiser attempting to cancel directly should have the action recorded as a cancellation request for the Coordinator to action</t>
         </is>
       </c>
-      <c r="G343" s="2" t="inlineStr">
+      <c r="G347" s="2" t="inlineStr">
         <is>
           <t>Event "Community Meetup" has status "Confirmed", assigned to coordinator_1@connectsphere.com</t>
         </is>
       </c>
-      <c r="H343" s="2" t="inlineStr">
+      <c r="H347" s="2" t="inlineStr">
         <is>
           <t>1. Log in as organiser_a@clienta.com
   2. Open event "Community Meetup"
@@ -18392,207 +18597,207 @@
   4. Enter a reason and submit</t>
         </is>
       </c>
-      <c r="I343" s="2" t="inlineStr">
+      <c r="I347" s="2" t="inlineStr">
         <is>
           <t>Reason: "No longer needed"</t>
         </is>
       </c>
-      <c r="J343" s="2" t="inlineStr">
+      <c r="J347" s="2" t="inlineStr">
         <is>
           <t>The event is NOT immediately cancelled; instead, a cancellation request is recorded and coordinator_1@connectsphere.com is notified to action it</t>
         </is>
       </c>
     </row>
-    <row r="344">
-      <c r="A344" s="2" t="n">
+    <row r="348">
+      <c r="A348" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="B344" s="2" t="inlineStr">
+      <c r="B348" s="2" t="inlineStr">
         <is>
           <t>E10-S04</t>
         </is>
       </c>
-      <c r="C344" s="2" t="inlineStr">
+      <c r="C348" s="2" t="inlineStr">
         <is>
           <t>E10-S04 - Scenario 5 (Pending change requests become Obsolete); C-77/T-88</t>
         </is>
       </c>
-      <c r="D344" s="2" t="inlineStr">
+      <c r="D348" s="2" t="inlineStr">
         <is>
           <t>3 - Integration / regression</t>
         </is>
       </c>
-      <c r="E344" s="2" t="inlineStr">
+      <c r="E348" s="2" t="inlineStr">
         <is>
           <t>TC_E10S04_06</t>
         </is>
       </c>
-      <c r="F344" s="2" t="inlineStr">
+      <c r="F348" s="2" t="inlineStr">
         <is>
           <t>Cancelling an Event should close every Pending change request as Obsolete</t>
         </is>
       </c>
-      <c r="G344" s="2" t="inlineStr">
+      <c r="G348" s="2" t="inlineStr">
         <is>
           <t>Event E-1 has two Pending change requests before cancellation</t>
         </is>
       </c>
-      <c r="H344" s="2" t="inlineStr">
+      <c r="H348" s="2" t="inlineStr">
         <is>
           <t>1. Cancel Event E-1 with a reason
 2. Inspect both change requests and history</t>
         </is>
       </c>
-      <c r="I344" s="2" t="inlineStr">
+      <c r="I348" s="2" t="inlineStr">
         <is>
           <t>Pending requests: CR-1, CR-2</t>
         </is>
       </c>
-      <c r="J344" s="2" t="inlineStr">
+      <c r="J348" s="2" t="inlineStr">
         <is>
           <t>Both requests become Obsolete automatically and each transition is recorded; neither is labelled rejected</t>
         </is>
       </c>
     </row>
-    <row r="345">
-      <c r="A345" s="2" t="n">
+    <row r="349">
+      <c r="A349" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B345" s="2" t="inlineStr">
+      <c r="B349" s="2" t="inlineStr">
         <is>
           <t>E10-S05</t>
         </is>
       </c>
-      <c r="C345" s="2" t="inlineStr">
+      <c r="C349" s="2" t="inlineStr">
         <is>
           <t>E10-S05 — Scenario 1 (Lost venue flags the event); C-120, T-81</t>
         </is>
       </c>
-      <c r="D345" s="2" t="inlineStr">
+      <c r="D349" s="2" t="inlineStr">
         <is>
           <t>2 - Happy Path</t>
         </is>
       </c>
-      <c r="E345" s="2" t="inlineStr">
+      <c r="E349" s="2" t="inlineStr">
         <is>
           <t>TC_E10S05_01</t>
         </is>
       </c>
-      <c r="F345" s="2" t="inlineStr">
+      <c r="F349" s="2" t="inlineStr">
         <is>
           <t>Verify that when a booked venue is marked unavailable the Coordinator's event should be flagged with the booking shown as Conflicting, return to Planning without being cancelled, and keep its other arrangements</t>
         </is>
       </c>
-      <c r="G345" s="2" t="inlineStr">
+      <c r="G349" s="2" t="inlineStr">
         <is>
           <t>Event "Charity Run" is Confirmed with a Confirmed booking at "Riverside Hall" on 15/01/2027 10:00-12:00, a reserved projector and an assigned technical staff member; coordinator_1@connectsphere.com owns it</t>
         </is>
       </c>
-      <c r="H345" s="2" t="inlineStr">
+      <c r="H349" s="2" t="inlineStr">
         <is>
           <t>1. As venue_staff_1@connectsphere.com, mark "Riverside Hall" unavailable 15/01/2027 00:00 to 16/01/2027 00:00, category "Renovation" (E05-S06)
   2. Sign in as coordinator_1@connectsphere.com and open the inbox
   3. Open event "Charity Run"</t>
         </is>
       </c>
-      <c r="I345" s="2" t="inlineStr">
+      <c r="I349" s="2" t="inlineStr">
         <is>
           <t>Event status before: Confirmed | Equipment: 1 projector reserved | Technical staff: 1 assigned</t>
         </is>
       </c>
-      <c r="J345" s="2" t="inlineStr">
+      <c r="J349" s="2" t="inlineStr">
         <is>
           <t>coordinator_1 has a notification about the lost venue; the event page shows a "needs alternative arrangements" flag with reason "Renovation", the venue booking marked Conflicting, status Planning (not Cancelled), and the projector reservation and staff assignment unchanged</t>
         </is>
       </c>
     </row>
-    <row r="346">
-      <c r="A346" s="2" t="n">
+    <row r="350">
+      <c r="A350" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B346" s="2" t="inlineStr">
+      <c r="B350" s="2" t="inlineStr">
         <is>
           <t>E10-S05</t>
         </is>
       </c>
-      <c r="C346" s="2" t="inlineStr">
+      <c r="C350" s="2" t="inlineStr">
         <is>
           <t>E10-S05 — Scenario 2 (Flagged event offers a replacement search)</t>
         </is>
       </c>
-      <c r="D346" s="2" t="inlineStr">
+      <c r="D350" s="2" t="inlineStr">
         <is>
           <t>2 - Happy Path</t>
         </is>
       </c>
-      <c r="E346" s="2" t="inlineStr">
+      <c r="E350" s="2" t="inlineStr">
         <is>
           <t>TC_E10S05_02</t>
         </is>
       </c>
-      <c r="F346" s="2" t="inlineStr">
+      <c r="F350" s="2" t="inlineStr">
         <is>
           <t>Verify that a flagged event should show the reason, period and affected booking, preserve the original event information, and offer a venue search for the same event</t>
         </is>
       </c>
-      <c r="G346" s="2" t="inlineStr">
+      <c r="G350" s="2" t="inlineStr">
         <is>
           <t>As TC_E10S05_01 after step 1; coordinator_1@connectsphere.com is signed in</t>
         </is>
       </c>
-      <c r="H346" s="2" t="inlineStr">
+      <c r="H350" s="2" t="inlineStr">
         <is>
           <t>1. Open event "Charity Run"
   2. Read the flag panel
   3. Click "Find a replacement venue"</t>
         </is>
       </c>
-      <c r="I346" s="2" t="inlineStr">
+      <c r="I350" s="2" t="inlineStr">
         <is>
           <t>Original: Riverside Hall, 15/01/2027 10:00-12:00, 120 attendees, Theatre layout, wheelchair access required</t>
         </is>
       </c>
-      <c r="J346" s="2" t="inlineStr">
+      <c r="J350" s="2" t="inlineStr">
         <is>
           <t>The panel shows reason "Renovation", period 15/01/2027, and the Conflicting Riverside Hall booking; the event's dates, attendance, layout and accessibility requirements are unchanged; the search opens pre-filled with those requirements for the same event (E06-S01)</t>
         </is>
       </c>
     </row>
-    <row r="347">
-      <c r="A347" s="2" t="n">
+    <row r="351">
+      <c r="A351" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B347" s="2" t="inlineStr">
+      <c r="B351" s="2" t="inlineStr">
         <is>
           <t>E10-S05</t>
         </is>
       </c>
-      <c r="C347" s="2" t="inlineStr">
+      <c r="C351" s="2" t="inlineStr">
         <is>
           <t>E10-S05 — Scenario 3 (Replacement requested without losing the original)</t>
         </is>
       </c>
-      <c r="D347" s="2" t="inlineStr">
+      <c r="D351" s="2" t="inlineStr">
         <is>
           <t>2 - Happy Path</t>
         </is>
       </c>
-      <c r="E347" s="2" t="inlineStr">
+      <c r="E351" s="2" t="inlineStr">
         <is>
           <t>TC_E10S05_03</t>
         </is>
       </c>
-      <c r="F347" s="2" t="inlineStr">
+      <c r="F351" s="2" t="inlineStr">
         <is>
           <t>Verify that requesting a replacement venue should create a second booking request on the same event without cancelling the Conflicting booking, which the Coordinator cancels explicitly afterwards</t>
         </is>
       </c>
-      <c r="G347" s="2" t="inlineStr">
+      <c r="G351" s="2" t="inlineStr">
         <is>
           <t>As TC_E10S05_02; venue "Harbour Suite" is Free on 15/01/2027 and meets the requirements</t>
         </is>
       </c>
-      <c r="H347" s="2" t="inlineStr">
+      <c r="H351" s="2" t="inlineStr">
         <is>
           <t>1. From the replacement search, request "Harbour Suite" for 15/01/2027 10:00-12:00 (E06-S03)
   2. Open event "Charity Run" and read its venue bookings
@@ -18600,359 +18805,359 @@
   4. As coordinator_1, cancel the Conflicting Riverside Hall booking</t>
         </is>
       </c>
-      <c r="I347" s="2" t="inlineStr">
+      <c r="I351" s="2" t="inlineStr">
         <is>
           <t>Replacement: Harbour Suite 15/01/2027 10:00-12:00</t>
         </is>
       </c>
-      <c r="J347" s="2" t="inlineStr">
+      <c r="J351" s="2" t="inlineStr">
         <is>
           <t>After step 1 the event shows two bookings: Riverside Hall (Conflicting) and Harbour Suite (Pending); after step 3 Harbour Suite is Confirmed and Riverside Hall is still Conflicting, not auto-cancelled; after step 4 only Harbour Suite remains and the event is not cancelled; with its venue reconfirmed, the event follows E08-S04 Scenario 4 rather than returning straight to Confirmed</t>
         </is>
       </c>
     </row>
-    <row r="348">
-      <c r="A348" s="2" t="n">
+    <row r="352">
+      <c r="A352" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B348" s="2" t="inlineStr">
+      <c r="B352" s="2" t="inlineStr">
         <is>
           <t>E10-S05</t>
         </is>
       </c>
-      <c r="C348" s="2" t="inlineStr">
+      <c r="C352" s="2" t="inlineStr">
         <is>
           <t>E10-S05 — Scenario 4 (Organiser and Attendees told on the actual change); C-121, T-81</t>
         </is>
       </c>
-      <c r="D348" s="2" t="inlineStr">
+      <c r="D352" s="2" t="inlineStr">
         <is>
           <t>3 - Cross-cutting (notification consistency)</t>
         </is>
       </c>
-      <c r="E348" s="2" t="inlineStr">
+      <c r="E352" s="2" t="inlineStr">
         <is>
           <t>TC_E10S05_04</t>
         </is>
       </c>
-      <c r="F348" s="2" t="inlineStr">
+      <c r="F352" s="2" t="inlineStr">
         <is>
           <t>Verify that the Organiser and registered Attendees should be notified of the venue change only when the replacement is confirmed, not when the original venue is lost</t>
         </is>
       </c>
-      <c r="G348" s="2" t="inlineStr">
+      <c r="G352" s="2" t="inlineStr">
         <is>
           <t>As TC_E10S05_03 with the Organiser organiser_1@connectsphere.com and two registered Attendees; notification relay enabled against the intercepted provider</t>
         </is>
       </c>
-      <c r="H348" s="2" t="inlineStr">
+      <c r="H352" s="2" t="inlineStr">
         <is>
           <t>1. After the venue is marked unavailable (TC_E10S05_01 step 1), check the Organiser's and Attendees' inboxes and the intercepted emails
   2. After the Harbour Suite request is approved (TC_E10S05_03 step 3), check them again</t>
         </is>
       </c>
-      <c r="I348" s="2" t="inlineStr">
+      <c r="I352" s="2" t="inlineStr">
         <is>
           <t>Recipients at step 2: organiser_1, attendee_1, attendee_2</t>
         </is>
       </c>
-      <c r="J348" s="2" t="inlineStr">
+      <c r="J352" s="2" t="inlineStr">
         <is>
           <t>At step 1 none of the Organiser or Attendees has a notification about the venue; at step 2 each has exactly one notification naming the new venue "Harbour Suite" via the existing venue-change routing (E11-S01)</t>
         </is>
       </c>
     </row>
-    <row r="349">
-      <c r="A349" s="2" t="n">
+    <row r="353">
+      <c r="A353" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="B349" s="2" t="inlineStr">
+      <c r="B353" s="2" t="inlineStr">
         <is>
           <t>E11-S01</t>
         </is>
       </c>
-      <c r="C349" s="2" t="inlineStr">
+      <c r="C353" s="2" t="inlineStr">
         <is>
           <t>E11-S01 - Scenario 1 (Status change notified)</t>
         </is>
       </c>
-      <c r="D349" s="2" t="inlineStr">
+      <c r="D353" s="2" t="inlineStr">
         <is>
           <t>2 - Happy Path</t>
         </is>
       </c>
-      <c r="E349" s="2" t="inlineStr">
+      <c r="E353" s="2" t="inlineStr">
         <is>
           <t>TC_E11S01_01</t>
         </is>
       </c>
-      <c r="F349" s="2" t="inlineStr">
+      <c r="F353" s="2" t="inlineStr">
         <is>
           <t>Verify that a user linked to an event should be notified when its status changes or a booking decision is made, with details of what/when/which event</t>
         </is>
       </c>
-      <c r="G349" s="2" t="inlineStr">
+      <c r="G353" s="2" t="inlineStr">
         <is>
           <t>organiser_a@clienta.com is linked to event "Annual Tech Summit", currently "Under Review"</t>
         </is>
       </c>
-      <c r="H349" s="2" t="inlineStr">
+      <c r="H353" s="2" t="inlineStr">
         <is>
           <t>1. As coordinator_1@connectsphere.com, approve request "Annual Tech Summit" (status -&gt; Approved)
   2. Log in as organiser_a@clienta.com and open notifications</t>
         </is>
       </c>
-      <c r="I349" s="2" t="inlineStr">
+      <c r="I353" s="2" t="inlineStr">
         <is>
           <t>Event: Annual Tech Summit | Change: Under Review -&gt; Approved</t>
         </is>
       </c>
-      <c r="J349" s="2" t="inlineStr">
+      <c r="J353" s="2" t="inlineStr">
         <is>
           <t>A notification is received stating the status changed to "Approved", the time of the change, and that it concerns "Annual Tech Summit"</t>
         </is>
       </c>
     </row>
-    <row r="350">
-      <c r="A350" s="2" t="n">
+    <row r="354">
+      <c r="A354" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="B350" s="2" t="inlineStr">
+      <c r="B354" s="2" t="inlineStr">
         <is>
           <t>E11-S01</t>
         </is>
       </c>
-      <c r="C350" s="2" t="inlineStr">
+      <c r="C354" s="2" t="inlineStr">
         <is>
           <t>E11-S01 - Scenario 2 (All affected parties notified)</t>
         </is>
       </c>
-      <c r="D350" s="2" t="inlineStr">
+      <c r="D354" s="2" t="inlineStr">
         <is>
           <t>2 - Happy Path</t>
         </is>
       </c>
-      <c r="E350" s="2" t="inlineStr">
+      <c r="E354" s="2" t="inlineStr">
         <is>
           <t>TC_E11S01_02</t>
         </is>
       </c>
-      <c r="F350" s="2" t="inlineStr">
+      <c r="F354" s="2" t="inlineStr">
         <is>
           <t>Verify that effective date, time or venue changes follow the approved recipient matrix</t>
         </is>
       </c>
-      <c r="G350" s="2" t="inlineStr">
+      <c r="G354" s="2" t="inlineStr">
         <is>
           <t>Event "Annual Tech Summit" the event has organiser_a@clienta.com, venue_staff_1@connectsphere.com, and tech_support_1@connectsphere.com assigned, and attendee_a@example.com registered; attendee_b@example.com is waitlisted and coordinator_1@connectsphere.com is the assigned Coordinator</t>
         </is>
       </c>
-      <c r="H350" s="2" t="inlineStr">
+      <c r="H354" s="2" t="inlineStr">
         <is>
           <t>1. As coordinator_1@connectsphere.com, change the event's venue
   2. Check notifications for organiser_a@clienta.com, venue_staff_1@connectsphere.com, tech_support_1@connectsphere.com, and attendee_a@example.com</t>
         </is>
       </c>
-      <c r="I350" s="2" t="inlineStr">
+      <c r="I354" s="2" t="inlineStr">
         <is>
           <t>Changed field: Venue</t>
         </is>
       </c>
-      <c r="J350" s="2" t="inlineStr">
+      <c r="J354" s="2" t="inlineStr">
         <is>
           <t>The Organiser, assigned Venue Staff, assigned Technical Support Staff, registered Attendee and waitlisted Attendee receive a notification. The acting Coordinator receives no self-notification. If another authorized actor or a system operation makes the change, the assigned Coordinator is included. Venue-move tests include responsible staff for both the old and new venues. Backend resolver fixtures are not evidence that the venue-assignment workflow is implemented.</t>
         </is>
       </c>
     </row>
-    <row r="351">
-      <c r="A351" s="2" t="n">
+    <row r="355">
+      <c r="A355" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="B351" s="2" t="inlineStr">
+      <c r="B355" s="2" t="inlineStr">
         <is>
           <t>E11-S01</t>
         </is>
       </c>
-      <c r="C351" s="2" t="inlineStr">
+      <c r="C355" s="2" t="inlineStr">
         <is>
           <t>E11-S01 - Scenario 3 (Unaffected users not notified)</t>
         </is>
       </c>
-      <c r="D351" s="2" t="inlineStr">
+      <c r="D355" s="2" t="inlineStr">
         <is>
           <t>4 - Negative</t>
         </is>
       </c>
-      <c r="E351" s="2" t="inlineStr">
+      <c r="E355" s="2" t="inlineStr">
         <is>
           <t>TC_E11S01_03</t>
         </is>
       </c>
-      <c r="F351" s="2" t="inlineStr">
+      <c r="F355" s="2" t="inlineStr">
         <is>
           <t>Verify that a user whose responsibilities are unaffected by a change should not be notified</t>
         </is>
       </c>
-      <c r="G351" s="2" t="inlineStr">
+      <c r="G355" s="2" t="inlineStr">
         <is>
           <t>Event "Annual Tech Summit" the event's Description field is about to be edited; venue_staff_1@connectsphere.com has no responsibility tied to the Description field</t>
         </is>
       </c>
-      <c r="H351" s="2" t="inlineStr">
+      <c r="H355" s="2" t="inlineStr">
         <is>
           <t>1. As organiser_a@clienta.com, edit the Description field only
   2. Check venue_staff_1@connectsphere.com's notifications</t>
         </is>
       </c>
-      <c r="I351" s="2" t="inlineStr">
+      <c r="I355" s="2" t="inlineStr">
         <is>
           <t>Changed field: Description only</t>
         </is>
       </c>
-      <c r="J351" s="2" t="inlineStr">
+      <c r="J355" s="2" t="inlineStr">
         <is>
           <t>venue_staff_1@connectsphere.com receives no notification, since the Description change does not affect their responsibilities</t>
         </is>
       </c>
     </row>
-    <row r="352">
-      <c r="A352" s="2" t="n">
+    <row r="356">
+      <c r="A356" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="B352" s="2" t="inlineStr">
+      <c r="B356" s="2" t="inlineStr">
         <is>
           <t>E11-S01</t>
         </is>
       </c>
-      <c r="C352" s="2" t="inlineStr">
+      <c r="C356" s="2" t="inlineStr">
         <is>
           <t>E11-S01 - Scenario 4 (Delivered in-app and by email)</t>
         </is>
       </c>
-      <c r="D352" s="2" t="inlineStr">
+      <c r="D356" s="2" t="inlineStr">
         <is>
           <t>2 - Happy Path</t>
         </is>
       </c>
-      <c r="E352" s="2" t="inlineStr">
+      <c r="E356" s="2" t="inlineStr">
         <is>
           <t>TC_E11S01_05</t>
         </is>
       </c>
-      <c r="F352" s="2" t="inlineStr">
+      <c r="F356" s="2" t="inlineStr">
         <is>
           <t>Verify that a generated notification should appear in the system and also be sent to the user's registered email address</t>
         </is>
       </c>
-      <c r="G352" s="2" t="inlineStr">
+      <c r="G356" s="2" t="inlineStr">
         <is>
           <t>organiser_a@clienta.com's registered email is organiser_a@clienta.com; a notification-triggering status change is about to occur on their event</t>
         </is>
       </c>
-      <c r="H352" s="2" t="inlineStr">
+      <c r="H356" s="2" t="inlineStr">
         <is>
           <t>1. Trigger a status change on organiser_a@clienta.com's event
   2. Log in as organiser_a@clienta.com and check the in-app notification list
   3. Check the inbox for organiser_a@clienta.com</t>
         </is>
       </c>
-      <c r="I352" s="2" t="inlineStr">
+      <c r="I356" s="2" t="inlineStr">
         <is>
           <t>Registered email: organiser_a@clienta.com</t>
         </is>
       </c>
-      <c r="J352" s="2" t="inlineStr">
+      <c r="J356" s="2" t="inlineStr">
         <is>
           <t>The notification appears in the in-app notification list, and an equivalent email is also delivered to organiser_a@clienta.com's inbox</t>
         </is>
       </c>
     </row>
-    <row r="353">
-      <c r="A353" s="2" t="n">
+    <row r="357">
+      <c r="A357" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="B353" s="2" t="inlineStr">
+      <c r="B357" s="2" t="inlineStr">
         <is>
           <t>E11-S01</t>
         </is>
       </c>
-      <c r="C353" s="2" t="inlineStr">
+      <c r="C357" s="2" t="inlineStr">
         <is>
           <t>E11-S01 - Scenario 5 (Unread notifications distinguished)</t>
         </is>
       </c>
-      <c r="D353" s="2" t="inlineStr">
+      <c r="D357" s="2" t="inlineStr">
         <is>
           <t>2 - Happy Path</t>
         </is>
       </c>
-      <c r="E353" s="2" t="inlineStr">
+      <c r="E357" s="2" t="inlineStr">
         <is>
           <t>TC_E11S01_06</t>
         </is>
       </c>
-      <c r="F353" s="2" t="inlineStr">
+      <c r="F357" s="2" t="inlineStr">
         <is>
           <t>Verify that opening the notification list with several unread notifications should show them newest first with unread ones distinguished</t>
         </is>
       </c>
-      <c r="G353" s="2" t="inlineStr">
+      <c r="G357" s="2" t="inlineStr">
         <is>
           <t>organiser_a@clienta.com has 3 notifications on 09/09/2026: 08:00 (read), 10:00 (unread), 14:00 (unread)</t>
         </is>
       </c>
-      <c r="H353" s="2" t="inlineStr">
+      <c r="H357" s="2" t="inlineStr">
         <is>
           <t>1. Log in as organiser_a@clienta.com
   2. Open the notification list</t>
         </is>
       </c>
-      <c r="I353" s="2" t="inlineStr">
+      <c r="I357" s="2" t="inlineStr">
         <is>
           <t>Notifications: 08:00 (read), 10:00 (unread), 14:00 (unread)</t>
         </is>
       </c>
-      <c r="J353" s="2" t="inlineStr">
+      <c r="J357" s="2" t="inlineStr">
         <is>
           <t>Notifications are listed newest first (14:00, then 10:00, then 08:00), with the 14:00 and 10:00 entries visually marked as unread and 08:00 shown as read</t>
         </is>
       </c>
     </row>
-    <row r="354">
-      <c r="A354" s="2" t="n">
+    <row r="358">
+      <c r="A358" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="B354" s="2" t="inlineStr">
+      <c r="B358" s="2" t="inlineStr">
         <is>
           <t>E11-S01</t>
         </is>
       </c>
-      <c r="C354" s="2" t="inlineStr">
+      <c r="C358" s="2" t="inlineStr">
         <is>
           <t>E11-S01 - Scenario 6 (Marked as read)</t>
         </is>
       </c>
-      <c r="D354" s="2" t="inlineStr">
+      <c r="D358" s="2" t="inlineStr">
         <is>
           <t>2 - Happy Path</t>
         </is>
       </c>
-      <c r="E354" s="2" t="inlineStr">
+      <c r="E358" s="2" t="inlineStr">
         <is>
           <t>TC_E11S01_07</t>
         </is>
       </c>
-      <c r="F354" s="2" t="inlineStr">
+      <c r="F358" s="2" t="inlineStr">
         <is>
           <t>Verify that opening an unread notification should mark it as read</t>
         </is>
       </c>
-      <c r="G354" s="2" t="inlineStr">
+      <c r="G358" s="2" t="inlineStr">
         <is>
           <t>organiser_a@clienta.com has an unread notification from 10:00 on 09/09/2026</t>
         </is>
       </c>
-      <c r="H354" s="2" t="inlineStr">
+      <c r="H358" s="2" t="inlineStr">
         <is>
           <t>1. Log in as organiser_a@clienta.com
   2. Open the notification list
@@ -18960,52 +19165,52 @@
   4. Return to the notification list</t>
         </is>
       </c>
-      <c r="I354" s="2" t="inlineStr">
+      <c r="I358" s="2" t="inlineStr">
         <is>
           <t>Notification: 10:00 on 09/09/2026 (initially unread)</t>
         </is>
       </c>
-      <c r="J354" s="2" t="inlineStr">
+      <c r="J358" s="2" t="inlineStr">
         <is>
           <t>The 10:00 notification is now shown as read (no longer marked unread) in the list</t>
         </is>
       </c>
     </row>
-    <row r="355">
-      <c r="A355" s="2" t="n">
+    <row r="359">
+      <c r="A359" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="B355" s="2" t="inlineStr">
+      <c r="B359" s="2" t="inlineStr">
         <is>
           <t>E11-S01</t>
         </is>
       </c>
-      <c r="C355" s="2" t="inlineStr">
+      <c r="C359" s="2" t="inlineStr">
         <is>
           <t>E11-S01 · Scenario 5 (Delivered in-app and by email) · ADR-006</t>
         </is>
       </c>
-      <c r="D355" s="2" t="inlineStr">
+      <c r="D359" s="2" t="inlineStr">
         <is>
           <t>4 - Negative (third-party unavailable)</t>
         </is>
       </c>
-      <c r="E355" s="2" t="inlineStr">
+      <c r="E359" s="2" t="inlineStr">
         <is>
           <t>TC_E11S01_08</t>
         </is>
       </c>
-      <c r="F355" s="2" t="inlineStr">
+      <c r="F359" s="2" t="inlineStr">
         <is>
           <t>Verify that an unreachable email provider does not affect the business change or the in-app notification</t>
         </is>
       </c>
-      <c r="G355" s="2" t="inlineStr">
+      <c r="G359" s="2" t="inlineStr">
         <is>
           <t>Event EVT-2003 has an assigned Coordinator coord_a@connectsphere.com. The email provider endpoint is configured to an unreachable host so every SMTP attempt fails</t>
         </is>
       </c>
-      <c r="H355" s="2" t="inlineStr">
+      <c r="H359" s="2" t="inlineStr">
         <is>
           <t>1. Sign in as Venue Staff and approve the pending venue booking for EVT-2003
  2. Confirm the booking status has changed
@@ -19013,52 +19218,52 @@
  4. Inspect the delivery records for that notification</t>
         </is>
       </c>
-      <c r="I355" s="2" t="inlineStr">
+      <c r="I359" s="2" t="inlineStr">
         <is>
           <t>SMTP host: unreachable · Notification: venue booking approved</t>
         </is>
       </c>
-      <c r="J355" s="2" t="inlineStr">
+      <c r="J359" s="2" t="inlineStr">
         <is>
           <t>The booking is Confirmed and the change persists. The in-app notification appears for the Coordinator. The email delivery row is marked failed with a recorded reason. The business transaction is not rolled back by the email failure</t>
         </is>
       </c>
     </row>
-    <row r="356">
-      <c r="A356" s="2" t="n">
+    <row r="360">
+      <c r="A360" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="B356" s="2" t="inlineStr">
+      <c r="B360" s="2" t="inlineStr">
         <is>
           <t>E11-S01</t>
         </is>
       </c>
-      <c r="C356" s="2" t="inlineStr">
+      <c r="C360" s="2" t="inlineStr">
         <is>
           <t>E11-S01 · Scenario 1 (Status change notified) · ADR-006 outbox guarantee</t>
         </is>
       </c>
-      <c r="D356" s="2" t="inlineStr">
+      <c r="D360" s="2" t="inlineStr">
         <is>
           <t>4 - Negative (transaction rollback)</t>
         </is>
       </c>
-      <c r="E356" s="2" t="inlineStr">
+      <c r="E360" s="2" t="inlineStr">
         <is>
           <t>TC_E11S01_09</t>
         </is>
       </c>
-      <c r="F356" s="2" t="inlineStr">
+      <c r="F360" s="2" t="inlineStr">
         <is>
           <t>Verify that a rolled-back business transaction publishes no notification</t>
         </is>
       </c>
-      <c r="G356" s="2" t="inlineStr">
+      <c r="G360" s="2" t="inlineStr">
         <is>
           <t>Event EVT-2004 is at status Under Review. A fault is injected so that the approval transaction fails after the notification delivery rows are written but before commit</t>
         </is>
       </c>
-      <c r="H356" s="2" t="inlineStr">
+      <c r="H360" s="2" t="inlineStr">
         <is>
           <t>1. Sign in as the assigned Event Coordinator
  2. Approve EVT-2004, triggering the injected failure
@@ -19066,214 +19271,14 @@
  4. Inspect the job queue and the Organiser's notification list</t>
         </is>
       </c>
-      <c r="I356" s="2" t="inlineStr">
+      <c r="I360" s="2" t="inlineStr">
         <is>
           <t>Event: EVT-2004 · Injected failure point: after delivery rows written, before commit</t>
         </is>
       </c>
-      <c r="J356" s="2" t="inlineStr">
+      <c r="J360" s="2" t="inlineStr">
         <is>
           <t>The event remains at Under Review. No delivery row is persisted, nothing is published to the queue, and the Organiser receives no in-app notification and no email. Only committed deliveries are ever published</t>
-        </is>
-      </c>
-    </row>
-    <row r="357">
-      <c r="A357" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B357" s="2" t="inlineStr">
-        <is>
-          <t>E11-S01</t>
-        </is>
-      </c>
-      <c r="C357" s="2" t="inlineStr">
-        <is>
-          <t>E11-S01 - approved routing extension (T-64); ADR-006</t>
-        </is>
-      </c>
-      <c r="D357" s="2" t="inlineStr">
-        <is>
-          <t>3 - Integration / regression</t>
-        </is>
-      </c>
-      <c r="E357" s="2" t="inlineStr">
-        <is>
-          <t>TC_E11S01_10</t>
-        </is>
-      </c>
-      <c r="F357" s="2" t="inlineStr">
-        <is>
-          <t>Apply the approved role/change recipient matrix</t>
-        </is>
-      </c>
-      <c r="G357" s="2" t="inlineStr">
-        <is>
-          <t>The event has active links to all six recipient groups and a public snapshot.</t>
-        </is>
-      </c>
-      <c r="H357" s="2" t="inlineStr">
-        <is>
-          <t>1. Trigger each internal status, booking, equipment, public status, arrangement, place-release and description-only change through the selector.</t>
-        </is>
-      </c>
-      <c r="I357" s="2" t="inlineStr">
-        <is>
-          <t>Synthetic linked-user fixtures in disposable PostgreSQL; no live email provider calls.</t>
-        </is>
-      </c>
-      <c r="J357" s="2" t="inlineStr">
-        <is>
-          <t>Recipient sets match the E11-S01 matrix; internal decisions do not reach Attendees; initial Planning differs from Confirmed-to-Planning.</t>
-        </is>
-      </c>
-    </row>
-    <row r="358">
-      <c r="A358" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B358" s="2" t="inlineStr">
-        <is>
-          <t>E11-S01</t>
-        </is>
-      </c>
-      <c r="C358" s="2" t="inlineStr">
-        <is>
-          <t>E11-S01 - approved routing extension (T-64); ADR-006</t>
-        </is>
-      </c>
-      <c r="D358" s="2" t="inlineStr">
-        <is>
-          <t>3 - Integration / regression</t>
-        </is>
-      </c>
-      <c r="E358" s="2" t="inlineStr">
-        <is>
-          <t>TC_E11S01_11</t>
-        </is>
-      </c>
-      <c r="F358" s="2" t="inlineStr">
-        <is>
-          <t>Suppress self-notifications and duplicate recipient links</t>
-        </is>
-      </c>
-      <c r="G358" s="2" t="inlineStr">
-        <is>
-          <t>A user is both the actor and a candidate recipient; duplicated staff links exist.</t>
-        </is>
-      </c>
-      <c r="H358" s="2" t="inlineStr">
-        <is>
-          <t>1. Select recipients for an arrangement change and an actor-made booking decision.</t>
-        </is>
-      </c>
-      <c r="I358" s="2" t="inlineStr">
-        <is>
-          <t>Synthetic linked-user fixtures in disposable PostgreSQL; no live email provider calls.</t>
-        </is>
-      </c>
-      <c r="J358" s="2" t="inlineStr">
-        <is>
-          <t>The actor receives no routine self-notification; every remaining user appears once; system changes have no excluded actor.</t>
-        </is>
-      </c>
-    </row>
-    <row r="359">
-      <c r="A359" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B359" s="2" t="inlineStr">
-        <is>
-          <t>E11-S01</t>
-        </is>
-      </c>
-      <c r="C359" s="2" t="inlineStr">
-        <is>
-          <t>E11-S01 - approved routing extension (T-64); ADR-006</t>
-        </is>
-      </c>
-      <c r="D359" s="2" t="inlineStr">
-        <is>
-          <t>3 - Integration / regression</t>
-        </is>
-      </c>
-      <c r="E359" s="2" t="inlineStr">
-        <is>
-          <t>TC_E11S01_12</t>
-        </is>
-      </c>
-      <c r="F359" s="2" t="inlineStr">
-        <is>
-          <t>Preserve before/after recipients during cancellation and venue moves</t>
-        </is>
-      </c>
-      <c r="G359" s="2" t="inlineStr">
-        <is>
-          <t>An event has active bookings, assigned staff, registered and waitlisted Attendees.</t>
-        </is>
-      </c>
-      <c r="H359" s="2" t="inlineStr">
-        <is>
-          <t>1. Capture its audience, release links during cancellation or replace the venue, then call the hook with both snapshots.</t>
-        </is>
-      </c>
-      <c r="I359" s="2" t="inlineStr">
-        <is>
-          <t>Synthetic linked-user fixtures in disposable PostgreSQL; no live email provider calls.</t>
-        </is>
-      </c>
-      <c r="J359" s="2" t="inlineStr">
-        <is>
-          <t>Cancellation notifies the pre-release audience. Venue moves include responsible staff at both venues. These are hook-contract tests until the owning workflows integrate.</t>
-        </is>
-      </c>
-    </row>
-    <row r="360">
-      <c r="A360" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B360" s="2" t="inlineStr">
-        <is>
-          <t>E11-S01</t>
-        </is>
-      </c>
-      <c r="C360" s="2" t="inlineStr">
-        <is>
-          <t>E11-S01 - approved routing extension (T-64); ADR-006</t>
-        </is>
-      </c>
-      <c r="D360" s="2" t="inlineStr">
-        <is>
-          <t>3 - Integration / regression</t>
-        </is>
-      </c>
-      <c r="E360" s="2" t="inlineStr">
-        <is>
-          <t>TC_E11S01_13</t>
-        </is>
-      </c>
-      <c r="F360" s="2" t="inlineStr">
-        <is>
-          <t>Expose missing Venue Staff assignments without an unsafe fallback</t>
-        </is>
-      </c>
-      <c r="G360" s="2" t="inlineStr">
-        <is>
-          <t>No explicit venue assignment adapter is available; a booking has a decided_by actor and unrelated Venue Staff accounts exist.</t>
-        </is>
-      </c>
-      <c r="H360" s="2" t="inlineStr">
-        <is>
-          <t>1. Capture the audience and select booking-request recipients.</t>
-        </is>
-      </c>
-      <c r="I360" s="2" t="inlineStr">
-        <is>
-          <t>Synthetic linked-user fixtures in disposable PostgreSQL; no live email provider calls.</t>
-        </is>
-      </c>
-      <c r="J360" s="2" t="inlineStr">
-        <is>
-          <t>Venue Staff recipients are unresolved, the venue IDs are reported, and neither decided_by nor all Venue Staff is substituted.</t>
         </is>
       </c>
     </row>
@@ -19298,22 +19303,22 @@
       </c>
       <c r="E361" s="2" t="inlineStr">
         <is>
-          <t>TC_E11S01_14</t>
+          <t>TC_E11S01_10</t>
         </is>
       </c>
       <c r="F361" s="2" t="inlineStr">
         <is>
-          <t>Protect attendee notification content and membership boundaries</t>
+          <t>Apply the approved role/change recipient matrix</t>
         </is>
       </c>
       <c r="G361" s="2" t="inlineStr">
         <is>
-          <t>The internal event title differs from its publication; registered, waitlisted, withdrawn, inactive and unrelated users exist.</t>
+          <t>The event has active links to all six recipient groups and a public snapshot.</t>
         </is>
       </c>
       <c r="H361" s="2" t="inlineStr">
         <is>
-          <t>1. Apply an effective date change; inspect notification messages and retained email payloads. Also select recipients for an unpublished event.</t>
+          <t>1. Trigger each internal status, booking, equipment, public status, arrangement, place-release and description-only change through the selector.</t>
         </is>
       </c>
       <c r="I361" s="2" t="inlineStr">
@@ -19323,7 +19328,7 @@
       </c>
       <c r="J361" s="2" t="inlineStr">
         <is>
-          <t>Only eligible linked active users are selected. Attendees receive the published event name and fixed public change description; no internal title/reason/comment leaks. Unpublished events produce no attendee notice.</t>
+          <t>Recipient sets match the E11-S01 matrix; internal decisions do not reach Attendees; initial Planning differs from Confirmed-to-Planning.</t>
         </is>
       </c>
     </row>
@@ -19348,22 +19353,22 @@
       </c>
       <c r="E362" s="2" t="inlineStr">
         <is>
-          <t>TC_E11S01_15</t>
+          <t>TC_E11S01_11</t>
         </is>
       </c>
       <c r="F362" s="2" t="inlineStr">
         <is>
-          <t>Deduplicate concurrent notification-hook retries</t>
+          <t>Suppress self-notifications and duplicate recipient links</t>
         </is>
       </c>
       <c r="G362" s="2" t="inlineStr">
         <is>
-          <t>Two transactions use the same event, stable change ID and recipient snapshot.</t>
+          <t>A user is both the actor and a candidate recipient; duplicated staff links exist.</t>
         </is>
       </c>
       <c r="H362" s="2" t="inlineStr">
         <is>
-          <t>1. Call the notification hook concurrently and commit both attempts.</t>
+          <t>1. Select recipients for an arrangement change and an actor-made booking decision.</t>
         </is>
       </c>
       <c r="I362" s="2" t="inlineStr">
@@ -19373,7 +19378,7 @@
       </c>
       <c r="J362" s="2" t="inlineStr">
         <is>
-          <t>Exactly one in-app row and one email-delivery row exist per recipient for the logical change. A new change ID identifies a different business change.</t>
+          <t>The actor receives no routine self-notification; every remaining user appears once; system changes have no excluded actor.</t>
         </is>
       </c>
     </row>
@@ -19398,22 +19403,22 @@
       </c>
       <c r="E363" s="2" t="inlineStr">
         <is>
-          <t>TC_E11S01_16</t>
+          <t>TC_E11S01_12</t>
         </is>
       </c>
       <c r="F363" s="2" t="inlineStr">
         <is>
-          <t>Keep uncommitted notifications invisible and roll back all writes</t>
+          <t>Preserve before/after recipients during cancellation and venue moves</t>
         </is>
       </c>
       <c r="G363" s="2" t="inlineStr">
         <is>
-          <t>A business transaction has inserted notifications and prepared email delivery rows but has not committed.</t>
+          <t>An event has active bookings, assigned staff, registered and waitlisted Attendees.</t>
         </is>
       </c>
       <c r="H363" s="2" t="inlineStr">
         <is>
-          <t>1. Read from another connection, then force the business transaction to roll back.</t>
+          <t>1. Capture its audience, release links during cancellation or replace the venue, then call the hook with both snapshots.</t>
         </is>
       </c>
       <c r="I363" s="2" t="inlineStr">
@@ -19423,45 +19428,245 @@
       </c>
       <c r="J363" s="2" t="inlineStr">
         <is>
-          <t>The other connection cannot observe the uncommitted messages. After rollback no notification or email-delivery row remains.</t>
+          <t>Cancellation notifies the pre-release audience. Venue moves include responsible staff at both venues. These are hook-contract tests until the owning workflows integrate.</t>
         </is>
       </c>
     </row>
     <row r="364">
       <c r="A364" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B364" s="2" t="inlineStr">
+        <is>
+          <t>E11-S01</t>
+        </is>
+      </c>
+      <c r="C364" s="2" t="inlineStr">
+        <is>
+          <t>E11-S01 - approved routing extension (T-64); ADR-006</t>
+        </is>
+      </c>
+      <c r="D364" s="2" t="inlineStr">
+        <is>
+          <t>3 - Integration / regression</t>
+        </is>
+      </c>
+      <c r="E364" s="2" t="inlineStr">
+        <is>
+          <t>TC_E11S01_13</t>
+        </is>
+      </c>
+      <c r="F364" s="2" t="inlineStr">
+        <is>
+          <t>Expose missing Venue Staff assignments without an unsafe fallback</t>
+        </is>
+      </c>
+      <c r="G364" s="2" t="inlineStr">
+        <is>
+          <t>No explicit venue assignment adapter is available; a booking has a decided_by actor and unrelated Venue Staff accounts exist.</t>
+        </is>
+      </c>
+      <c r="H364" s="2" t="inlineStr">
+        <is>
+          <t>1. Capture the audience and select booking-request recipients.</t>
+        </is>
+      </c>
+      <c r="I364" s="2" t="inlineStr">
+        <is>
+          <t>Synthetic linked-user fixtures in disposable PostgreSQL; no live email provider calls.</t>
+        </is>
+      </c>
+      <c r="J364" s="2" t="inlineStr">
+        <is>
+          <t>Venue Staff recipients are unresolved, the venue IDs are reported, and neither decided_by nor all Venue Staff is substituted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B365" s="2" t="inlineStr">
+        <is>
+          <t>E11-S01</t>
+        </is>
+      </c>
+      <c r="C365" s="2" t="inlineStr">
+        <is>
+          <t>E11-S01 - approved routing extension (T-64); ADR-006</t>
+        </is>
+      </c>
+      <c r="D365" s="2" t="inlineStr">
+        <is>
+          <t>3 - Integration / regression</t>
+        </is>
+      </c>
+      <c r="E365" s="2" t="inlineStr">
+        <is>
+          <t>TC_E11S01_14</t>
+        </is>
+      </c>
+      <c r="F365" s="2" t="inlineStr">
+        <is>
+          <t>Protect attendee notification content and membership boundaries</t>
+        </is>
+      </c>
+      <c r="G365" s="2" t="inlineStr">
+        <is>
+          <t>The internal event title differs from its publication; registered, waitlisted, withdrawn, inactive and unrelated users exist.</t>
+        </is>
+      </c>
+      <c r="H365" s="2" t="inlineStr">
+        <is>
+          <t>1. Apply an effective date change; inspect notification messages and retained email payloads. Also select recipients for an unpublished event.</t>
+        </is>
+      </c>
+      <c r="I365" s="2" t="inlineStr">
+        <is>
+          <t>Synthetic linked-user fixtures in disposable PostgreSQL; no live email provider calls.</t>
+        </is>
+      </c>
+      <c r="J365" s="2" t="inlineStr">
+        <is>
+          <t>Only eligible linked active users are selected. Attendees receive the published event name and fixed public change description; no internal title/reason/comment leaks. Unpublished events produce no attendee notice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B366" s="2" t="inlineStr">
+        <is>
+          <t>E11-S01</t>
+        </is>
+      </c>
+      <c r="C366" s="2" t="inlineStr">
+        <is>
+          <t>E11-S01 - approved routing extension (T-64); ADR-006</t>
+        </is>
+      </c>
+      <c r="D366" s="2" t="inlineStr">
+        <is>
+          <t>3 - Integration / regression</t>
+        </is>
+      </c>
+      <c r="E366" s="2" t="inlineStr">
+        <is>
+          <t>TC_E11S01_15</t>
+        </is>
+      </c>
+      <c r="F366" s="2" t="inlineStr">
+        <is>
+          <t>Deduplicate concurrent notification-hook retries</t>
+        </is>
+      </c>
+      <c r="G366" s="2" t="inlineStr">
+        <is>
+          <t>Two transactions use the same event, stable change ID and recipient snapshot.</t>
+        </is>
+      </c>
+      <c r="H366" s="2" t="inlineStr">
+        <is>
+          <t>1. Call the notification hook concurrently and commit both attempts.</t>
+        </is>
+      </c>
+      <c r="I366" s="2" t="inlineStr">
+        <is>
+          <t>Synthetic linked-user fixtures in disposable PostgreSQL; no live email provider calls.</t>
+        </is>
+      </c>
+      <c r="J366" s="2" t="inlineStr">
+        <is>
+          <t>Exactly one in-app row and one email-delivery row exist per recipient for the logical change. A new change ID identifies a different business change.</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B367" s="2" t="inlineStr">
+        <is>
+          <t>E11-S01</t>
+        </is>
+      </c>
+      <c r="C367" s="2" t="inlineStr">
+        <is>
+          <t>E11-S01 - approved routing extension (T-64); ADR-006</t>
+        </is>
+      </c>
+      <c r="D367" s="2" t="inlineStr">
+        <is>
+          <t>3 - Integration / regression</t>
+        </is>
+      </c>
+      <c r="E367" s="2" t="inlineStr">
+        <is>
+          <t>TC_E11S01_16</t>
+        </is>
+      </c>
+      <c r="F367" s="2" t="inlineStr">
+        <is>
+          <t>Keep uncommitted notifications invisible and roll back all writes</t>
+        </is>
+      </c>
+      <c r="G367" s="2" t="inlineStr">
+        <is>
+          <t>A business transaction has inserted notifications and prepared email delivery rows but has not committed.</t>
+        </is>
+      </c>
+      <c r="H367" s="2" t="inlineStr">
+        <is>
+          <t>1. Read from another connection, then force the business transaction to roll back.</t>
+        </is>
+      </c>
+      <c r="I367" s="2" t="inlineStr">
+        <is>
+          <t>Synthetic linked-user fixtures in disposable PostgreSQL; no live email provider calls.</t>
+        </is>
+      </c>
+      <c r="J367" s="2" t="inlineStr">
+        <is>
+          <t>The other connection cannot observe the uncommitted messages. After rollback no notification or email-delivery row remains.</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B364" s="2" t="inlineStr">
+      <c r="B368" s="2" t="inlineStr">
         <is>
           <t>E14-S02</t>
         </is>
       </c>
-      <c r="C364" s="2" t="inlineStr">
+      <c r="C368" s="2" t="inlineStr">
         <is>
           <t>E14-S02 - Scenario 1 (Status change recorded; T-75, T-76)</t>
         </is>
       </c>
-      <c r="D364" s="2" t="inlineStr">
+      <c r="D368" s="2" t="inlineStr">
         <is>
           <t>2 - Happy Path</t>
         </is>
       </c>
-      <c r="E364" s="2" t="inlineStr">
+      <c r="E368" s="2" t="inlineStr">
         <is>
           <t>TC_E14S02_01</t>
         </is>
       </c>
-      <c r="F364" s="2" t="inlineStr">
+      <c r="F368" s="2" t="inlineStr">
         <is>
           <t>Verify that an event status change should be recorded with the actor, action, affected event, and time</t>
         </is>
       </c>
-      <c r="G364" s="2" t="inlineStr">
+      <c r="G368" s="2" t="inlineStr">
         <is>
           <t>Request "Annual Tech Summit" has status "Under Review"; coordinator_1@connectsphere.com is an Event Coordinator permitted to view and approve it</t>
         </is>
       </c>
-      <c r="H364" s="2" t="inlineStr">
+      <c r="H368" s="2" t="inlineStr">
         <is>
           <t>1. As coordinator_1@connectsphere.com, approve the request (status -&gt; Approved)
 2. Open the approved event's existing detail page as that Coordinator
@@ -19469,52 +19674,52 @@
 4. Compare the displayed actor, action and timestamp with the completed change and affected event</t>
         </is>
       </c>
-      <c r="I364" s="2" t="inlineStr">
+      <c r="I368" s="2" t="inlineStr">
         <is>
           <t>Event: Annual Tech Summit | Action: Approve</t>
         </is>
       </c>
-      <c r="J364" s="2" t="inlineStr">
+      <c r="J368" s="2" t="inlineStr">
         <is>
           <t>An entry is recorded with actor = coordinator_1@connectsphere.com, action = "Status changed to Approved", event = Annual Tech Summit, and a timestamp; the Event Coordinator can read it on that event under existing access rules, without an Administrator role or global audit screen</t>
         </is>
       </c>
     </row>
-    <row r="365">
-      <c r="A365" s="2" t="n">
+    <row r="369">
+      <c r="A369" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B365" s="2" t="inlineStr">
+      <c r="B369" s="2" t="inlineStr">
         <is>
           <t>E14-S02</t>
         </is>
       </c>
-      <c r="C365" s="2" t="inlineStr">
+      <c r="C369" s="2" t="inlineStr">
         <is>
           <t>E14-S02 - Scenario 2 (Access denial recorded; T-75, T-76)</t>
         </is>
       </c>
-      <c r="D365" s="2" t="inlineStr">
+      <c r="D369" s="2" t="inlineStr">
         <is>
           <t>2 - Happy Path</t>
         </is>
       </c>
-      <c r="E365" s="2" t="inlineStr">
+      <c r="E369" s="2" t="inlineStr">
         <is>
           <t>TC_E14S02_02</t>
         </is>
       </c>
-      <c r="F365" s="2" t="inlineStr">
+      <c r="F369" s="2" t="inlineStr">
         <is>
           <t>Verify that a denied access attempt should be recorded with the user, target, and time</t>
         </is>
       </c>
-      <c r="G365" s="2" t="inlineStr">
+      <c r="G369" s="2" t="inlineStr">
         <is>
           <t>organiser_a@clienta.com is linked to Client A; event EVT-B01 belongs to Client B; the tester has read access to a controlled test database</t>
         </is>
       </c>
-      <c r="H365" s="2" t="inlineStr">
+      <c r="H369" s="2" t="inlineStr">
         <is>
           <t>1. As organiser_a@clienta.com, attempt to access EVT-B01 directly
 2. Confirm the request is refused
@@ -19522,155 +19727,155 @@
 4. Check the matching denial row's user, target, action and timestamp</t>
         </is>
       </c>
-      <c r="I365" s="2" t="inlineStr">
+      <c r="I369" s="2" t="inlineStr">
         <is>
           <t>User: organiser_a@clienta.com | Target: EVT-B01</t>
         </is>
       </c>
-      <c r="J365" s="2" t="inlineStr">
+      <c r="J369" s="2" t="inlineStr">
         <is>
           <t>An entry is recorded with user = organiser_a@clienta.com, target = EVT-B01, action = "Access Denied", and a timestamp</t>
         </is>
       </c>
     </row>
-    <row r="366">
-      <c r="A366" s="2" t="n">
+    <row r="370">
+      <c r="A370" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="B366" s="2" t="inlineStr">
+      <c r="B370" s="2" t="inlineStr">
         <is>
           <t>E14-S02</t>
         </is>
       </c>
-      <c r="C366" s="2" t="inlineStr">
+      <c r="C370" s="2" t="inlineStr">
         <is>
           <t>E14-S02 - former Scenario 3 (transferred to E06-S04 Scenario 5 by T-76; see TC_E06S04_05)</t>
         </is>
       </c>
-      <c r="D366" s="2" t="inlineStr">
+      <c r="D370" s="2" t="inlineStr">
         <is>
           <t>2 - Happy Path</t>
         </is>
       </c>
-      <c r="E366" s="2" t="inlineStr">
+      <c r="E370" s="2" t="inlineStr">
         <is>
           <t>TC_E14S02_03</t>
         </is>
       </c>
-      <c r="F366" s="2" t="inlineStr">
+      <c r="F370" s="2" t="inlineStr">
         <is>
           <t>[RETIRED — moved to TC_E06S04_05 by T-76] Verify that an approved venue booking should be recorded with the actor, action, affected records, and time</t>
         </is>
       </c>
-      <c r="G366" s="2" t="inlineStr">
+      <c r="G370" s="2" t="inlineStr">
         <is>
           <t>A booking request for Venue Z is pending</t>
         </is>
       </c>
-      <c r="H366" s="2" t="inlineStr">
+      <c r="H370" s="2" t="inlineStr">
         <is>
           <t>1. Do not execute this retired case; use TC_E06S04_05 under E06-S04 Scenario 5.
 2. Refer to the earlier dated workbook for the original steps.</t>
         </is>
       </c>
-      <c r="I366" s="2" t="inlineStr">
+      <c r="I370" s="2" t="inlineStr">
         <is>
           <t>Venue: Venue Z | Action: Approve Booking</t>
         </is>
       </c>
-      <c r="J366" s="2" t="inlineStr">
+      <c r="J370" s="2" t="inlineStr">
         <is>
           <t>An entry is recorded with the actor, action ("Booking Approved"), the affected booking/event, and a timestamp</t>
         </is>
       </c>
     </row>
-    <row r="367">
-      <c r="A367" s="2" t="n">
+    <row r="371">
+      <c r="A371" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B367" s="2" t="inlineStr">
+      <c r="B371" s="2" t="inlineStr">
         <is>
           <t>E14-S02</t>
         </is>
       </c>
-      <c r="C367" s="2" t="inlineStr">
+      <c r="C371" s="2" t="inlineStr">
         <is>
           <t>E14-S02 - Scenario 4 (Deactivation recorded; T-75, T-76)</t>
         </is>
       </c>
-      <c r="D367" s="2" t="inlineStr">
+      <c r="D371" s="2" t="inlineStr">
         <is>
           <t>2 - Happy Path</t>
         </is>
       </c>
-      <c r="E367" s="2" t="inlineStr">
+      <c r="E371" s="2" t="inlineStr">
         <is>
           <t>TC_E14S02_04</t>
         </is>
       </c>
-      <c r="F367" s="2" t="inlineStr">
+      <c r="F371" s="2" t="inlineStr">
         <is>
           <t>Verify that an account deactivation should be recorded in the activity log</t>
         </is>
       </c>
-      <c r="G367" s="2" t="inlineStr">
+      <c r="G371" s="2" t="inlineStr">
         <is>
           <t>organiser_a@clienta.com is signed in; the tester has read access to a controlled test database</t>
         </is>
       </c>
-      <c r="H367" s="2" t="inlineStr">
+      <c r="H371" s="2" t="inlineStr">
         <is>
           <t>1. As organiser_a@clienta.com, deactivate the account
 2. As the tester, query audit_logs in the controlled test database for that account and action time
 3. Check the matching deactivation row's actor, action and timestamp</t>
         </is>
       </c>
-      <c r="I367" s="2" t="inlineStr">
+      <c r="I371" s="2" t="inlineStr">
         <is>
           <t>Account: organiser_a@clienta.com</t>
         </is>
       </c>
-      <c r="J367" s="2" t="inlineStr">
+      <c r="J371" s="2" t="inlineStr">
         <is>
           <t>An entry is recorded showing the account deactivation with actor and timestamp</t>
         </is>
       </c>
     </row>
-    <row r="368">
-      <c r="A368" s="2" t="n">
+    <row r="372">
+      <c r="A372" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B368" s="2" t="inlineStr">
+      <c r="B372" s="2" t="inlineStr">
         <is>
           <t>E14-S02</t>
         </is>
       </c>
-      <c r="C368" s="2" t="inlineStr">
+      <c r="C372" s="2" t="inlineStr">
         <is>
           <t>E14-S02 - Scenario 5 (Log entries immutable; T-75, T-76)</t>
         </is>
       </c>
-      <c r="D368" s="2" t="inlineStr">
+      <c r="D372" s="2" t="inlineStr">
         <is>
           <t>4 - Negative</t>
         </is>
       </c>
-      <c r="E368" s="2" t="inlineStr">
+      <c r="E372" s="2" t="inlineStr">
         <is>
           <t>TC_E14S02_05</t>
         </is>
       </c>
-      <c r="F368" s="2" t="inlineStr">
+      <c r="F372" s="2" t="inlineStr">
         <is>
           <t>Verify that any attempt to edit or delete an activity log entry should be refused</t>
         </is>
       </c>
-      <c r="G368" s="2" t="inlineStr">
+      <c r="G372" s="2" t="inlineStr">
         <is>
           <t>A log entry exists: Event = Annual Tech Summit, Action = "Status changed to Approved", Actor = coordinator_1@connectsphere.com (created in TC_E14S02_01 or an equivalent independent fixture in a disposable test database)</t>
         </is>
       </c>
-      <c r="H368" s="2" t="inlineStr">
+      <c r="H372" s="2" t="inlineStr">
         <is>
           <t>1. As an Event Coordinator permitted to view the event, open its Activity log
 2. Confirm no edit or delete control is offered for the entry
@@ -19679,154 +19884,154 @@
 5. Read the original entry after each refused attempt to confirm its contents and row remain unchanged</t>
         </is>
       </c>
-      <c r="I368" s="2" t="inlineStr">
+      <c r="I372" s="2" t="inlineStr">
         <is>
           <t>Target log entry: Event = Annual Tech Summit, Action = "Status changed to Approved" | Attempted edit: Action -&gt; "Status changed to Rejected"</t>
         </is>
       </c>
-      <c r="J368" s="2" t="inlineStr">
+      <c r="J372" s="2" t="inlineStr">
         <is>
           <t>All update and delete attempts are refused. Unsupported API methods or routes may return 404/405; protected mutation routes must reject unauthorised requests. No response may represent a successful mutation. The database rejects both operations and the entry remains unchanged. No Administrator role is required.</t>
         </is>
       </c>
     </row>
-    <row r="369">
-      <c r="A369" s="2" t="n">
+    <row r="373">
+      <c r="A373" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="B369" s="2" t="inlineStr">
+      <c r="B373" s="2" t="inlineStr">
         <is>
           <t>E14-S02</t>
         </is>
       </c>
-      <c r="C369" s="2" t="inlineStr">
+      <c r="C373" s="2" t="inlineStr">
         <is>
           <t>E14-S02 - former Scenario 3 (transferred to E06-S04 Scenario 5 by T-76; see TC_E06S04_06)</t>
         </is>
       </c>
-      <c r="D369" s="2" t="inlineStr">
+      <c r="D373" s="2" t="inlineStr">
         <is>
           <t>2 - Happy Path</t>
         </is>
       </c>
-      <c r="E369" s="2" t="inlineStr">
+      <c r="E373" s="2" t="inlineStr">
         <is>
           <t>TC_E14S02_06</t>
         </is>
       </c>
-      <c r="F369" s="2" t="inlineStr">
+      <c r="F373" s="2" t="inlineStr">
         <is>
           <t>[RETIRED — moved to TC_E06S04_06 by T-76] Verify that a rejected venue booking should be recorded with the actor, action, affected records, and time</t>
         </is>
       </c>
-      <c r="G369" s="2" t="inlineStr">
+      <c r="G373" s="2" t="inlineStr">
         <is>
           <t>A booking request for Venue Z is pending</t>
         </is>
       </c>
-      <c r="H369" s="2" t="inlineStr">
+      <c r="H373" s="2" t="inlineStr">
         <is>
           <t>1. Do not execute this retired case; use TC_E06S04_06 under E06-S04 Scenario 5.
 2. Refer to the earlier dated workbook for the original steps.</t>
         </is>
       </c>
-      <c r="I369" s="2" t="inlineStr">
+      <c r="I373" s="2" t="inlineStr">
         <is>
           <t>Venue: Venue Z | Action: Reject Booking | Reason: Venue unavailable for maintenance</t>
         </is>
       </c>
-      <c r="J369" s="2" t="inlineStr">
+      <c r="J373" s="2" t="inlineStr">
         <is>
           <t>An entry is recorded with the actor, action ("Booking Rejected"), the affected booking/event, and a timestamp</t>
         </is>
       </c>
     </row>
-    <row r="370">
-      <c r="A370" s="2" t="n">
+    <row r="374">
+      <c r="A374" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="B370" s="2" t="inlineStr">
+      <c r="B374" s="2" t="inlineStr">
         <is>
           <t>E14-S02</t>
         </is>
       </c>
-      <c r="C370" s="2" t="inlineStr">
+      <c r="C374" s="2" t="inlineStr">
         <is>
           <t>E14-S02 - former Scenario 3 (transferred to E06-S04 Scenario 5 by T-76; see TC_E06S04_07)</t>
         </is>
       </c>
-      <c r="D370" s="2" t="inlineStr">
+      <c r="D374" s="2" t="inlineStr">
         <is>
           <t>2 - Happy Path</t>
         </is>
       </c>
-      <c r="E370" s="2" t="inlineStr">
+      <c r="E374" s="2" t="inlineStr">
         <is>
           <t>TC_E14S02_07</t>
         </is>
       </c>
-      <c r="F370" s="2" t="inlineStr">
+      <c r="F374" s="2" t="inlineStr">
         <is>
           <t>[RETIRED — moved to TC_E06S04_07 by T-76] Verify that a released venue booking should be recorded with the actor, action, affected records, and time</t>
         </is>
       </c>
-      <c r="G370" s="2" t="inlineStr">
+      <c r="G374" s="2" t="inlineStr">
         <is>
           <t>Venue Z has a confirmed booking for event "Annual Tech Summit"</t>
         </is>
       </c>
-      <c r="H370" s="2" t="inlineStr">
+      <c r="H374" s="2" t="inlineStr">
         <is>
           <t>1. Do not execute this retired case; use TC_E06S04_07 under E06-S04 Scenario 5.
 2. Refer to the earlier dated workbook for the original steps.</t>
         </is>
       </c>
-      <c r="I370" s="2" t="inlineStr">
+      <c r="I374" s="2" t="inlineStr">
         <is>
           <t>Venue: Venue Z | Action: Release Booking | Event: Annual Tech Summit</t>
         </is>
       </c>
-      <c r="J370" s="2" t="inlineStr">
+      <c r="J374" s="2" t="inlineStr">
         <is>
           <t>An entry is recorded with the actor, action ("Booking Released"), the affected booking/event, and a timestamp</t>
         </is>
       </c>
     </row>
-    <row r="371">
-      <c r="A371" s="2" t="n">
+    <row r="375">
+      <c r="A375" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B371" s="2" t="inlineStr">
+      <c r="B375" s="2" t="inlineStr">
         <is>
           <t>E14-S02</t>
         </is>
       </c>
-      <c r="C371" s="2" t="inlineStr">
+      <c r="C375" s="2" t="inlineStr">
         <is>
           <t>E14-S02 - Scenario 1 (Status change recorded; access-denial entries not shown; T-75)</t>
         </is>
       </c>
-      <c r="D371" s="2" t="inlineStr">
+      <c r="D375" s="2" t="inlineStr">
         <is>
           <t>3 - Cross-cutting (data isolation)</t>
         </is>
       </c>
-      <c r="E371" s="2" t="inlineStr">
+      <c r="E375" s="2" t="inlineStr">
         <is>
           <t>TC_E14S02_08</t>
         </is>
       </c>
-      <c r="F371" s="2" t="inlineStr">
+      <c r="F375" s="2" t="inlineStr">
         <is>
           <t>Verify that access-denial entries should not be shown in the event Activity log a Coordinator reads</t>
         </is>
       </c>
-      <c r="G371" s="2" t="inlineStr">
+      <c r="G375" s="2" t="inlineStr">
         <is>
           <t>Event EVT-2003 belongs to Client B, is Under Review and is assigned to coord_b@connectsphere.com; organiser_a@clienta.com belongs to Client A; the database is a disposable test database seeded with `npm run db:seed:test --workspace backend`</t>
         </is>
       </c>
-      <c r="H371" s="2" t="inlineStr">
+      <c r="H375" s="2" t="inlineStr">
         <is>
           <t>1. As organiser_a@clienta.com, attempt to open EVT-2003 directly and confirm the request is refused
 2. As the tester, confirm in the test database that an "Access Denied" row naming organiser_a@clienta.com now exists for that attempt
@@ -19835,52 +20040,52 @@
 5. Check every entry shown</t>
         </is>
       </c>
-      <c r="I371" s="2" t="inlineStr">
+      <c r="I375" s="2" t="inlineStr">
         <is>
           <t>Refused user: organiser_a@clienta.com (Organiser A, Client A) | Event: EVT-2003 (Client B) | Reader: coord_b@connectsphere.com</t>
         </is>
       </c>
-      <c r="J371" s="2" t="inlineStr">
+      <c r="J375" s="2" t="inlineStr">
         <is>
           <t>The Activity log shows the status-change entry from step 3 and no "Access Denied" entry; neither "Organiser A" nor organiser_a@clienta.com appears anywhere in the log</t>
         </is>
       </c>
     </row>
-    <row r="372">
-      <c r="A372" s="2" t="n">
+    <row r="376">
+      <c r="A376" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B372" s="2" t="inlineStr">
+      <c r="B376" s="2" t="inlineStr">
         <is>
           <t>E14-S03</t>
         </is>
       </c>
-      <c r="C372" s="2" t="inlineStr">
+      <c r="C376" s="2" t="inlineStr">
         <is>
           <t>E14-S03 - Scenario 1</t>
         </is>
       </c>
-      <c r="D372" s="2" t="inlineStr">
+      <c r="D376" s="2" t="inlineStr">
         <is>
           <t>2 - Happy Path</t>
         </is>
       </c>
-      <c r="E372" s="2" t="inlineStr">
+      <c r="E376" s="2" t="inlineStr">
         <is>
           <t>TC_E14S03_01</t>
         </is>
       </c>
-      <c r="F372" s="2" t="inlineStr">
+      <c r="F376" s="2" t="inlineStr">
         <is>
           <t>Organiser reads an edited date/time value in Singapore time</t>
         </is>
       </c>
-      <c r="G372" s="2" t="inlineStr">
+      <c r="G376" s="2" t="inlineStr">
         <is>
           <t>Planned, not executed. A disposable local event accessible to its Organiser has a controlled audit fixture for an edited startAt value; use the existing Organiser Activity log, not a new viewer.</t>
         </is>
       </c>
-      <c r="H372" s="2" t="inlineStr">
+      <c r="H376" s="2" t="inlineStr">
         <is>
           <t>1. Set the browser timezone to a non-Singapore timezone in the test environment.
 2. Sign in as the Organiser and open the event's Activity log.
@@ -19888,52 +20093,52 @@
 4. Reload and verify the displayed value remains the same.</t>
         </is>
       </c>
-      <c r="I372" s="2" t="inlineStr">
+      <c r="I376" s="2" t="inlineStr">
         <is>
           <t>field_changed: startAt; new_value: 2026-10-15T09:30:00Z; browser timezone: UTC.</t>
         </is>
       </c>
-      <c r="J372" s="2" t="inlineStr">
+      <c r="J376" s="2" t="inlineStr">
         <is>
           <t>The displayed edited value represents 15 October 2026 at 17:30 Singapore time (5:30 pm in the helper's format), on the same calendar date, not raw UTC or browser-local time. The Organiser view is not required to add a previously absent old-value display.</t>
         </is>
       </c>
     </row>
-    <row r="373">
-      <c r="A373" s="2" t="n">
+    <row r="377">
+      <c r="A377" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B373" s="2" t="inlineStr">
+      <c r="B377" s="2" t="inlineStr">
         <is>
           <t>E14-S03</t>
         </is>
       </c>
-      <c r="C373" s="2" t="inlineStr">
+      <c r="C377" s="2" t="inlineStr">
         <is>
           <t>E14-S03 - Scenario 1</t>
         </is>
       </c>
-      <c r="D373" s="2" t="inlineStr">
+      <c r="D377" s="2" t="inlineStr">
         <is>
           <t>2 - Happy Path</t>
         </is>
       </c>
-      <c r="E373" s="2" t="inlineStr">
+      <c r="E377" s="2" t="inlineStr">
         <is>
           <t>TC_E14S03_02</t>
         </is>
       </c>
-      <c r="F373" s="2" t="inlineStr">
+      <c r="F377" s="2" t="inlineStr">
         <is>
           <t>Assigned Coordinator reads existing before/after date/time values in Singapore time</t>
         </is>
       </c>
-      <c r="G373" s="2" t="inlineStr">
+      <c r="G377" s="2" t="inlineStr">
         <is>
           <t>Planned, not executed. A disposable event is accessible to its assigned Coordinator and has an edited date/time audit row whose existing Change cell shows old and new values.</t>
         </is>
       </c>
-      <c r="H373" s="2" t="inlineStr">
+      <c r="H377" s="2" t="inlineStr">
         <is>
           <t>1. Set the test browser timezone to UTC and open the assigned event as its Coordinator.
 2. Locate the edit in the existing Activity log Change column.
@@ -19941,52 +20146,52 @@
 4. Check that the existing actor and When columns still identify the same entry.</t>
         </is>
       </c>
-      <c r="I373" s="2" t="inlineStr">
+      <c r="I377" s="2" t="inlineStr">
         <is>
           <t>field_changed: startAt; old_value: 2026-10-15T08:30:00Z; new_value: 2026-10-15T09:30:00Z. This controlled historical fixture exercises an already-supported old/new display; it does not require the edit writer to start capturing new old values.</t>
         </is>
       </c>
-      <c r="J373" s="2" t="inlineStr">
+      <c r="J377" s="2" t="inlineStr">
         <is>
           <t>The existing before/after display represents 15 October at 16:30 -&gt; 17:30 Singapore time using the helper's formatting. No raw UTC strings remain for those edited date/time values; actor and occurrence timestamp semantics are unchanged.</t>
         </is>
       </c>
     </row>
-    <row r="374">
-      <c r="A374" s="2" t="n">
+    <row r="378">
+      <c r="A378" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B374" s="2" t="inlineStr">
+      <c r="B378" s="2" t="inlineStr">
         <is>
           <t>E14-S03</t>
         </is>
       </c>
-      <c r="C374" s="2" t="inlineStr">
+      <c r="C378" s="2" t="inlineStr">
         <is>
           <t>E14-S03 - Scenario 2</t>
         </is>
       </c>
-      <c r="D374" s="2" t="inlineStr">
+      <c r="D378" s="2" t="inlineStr">
         <is>
           <t>5 - Boundary</t>
         </is>
       </c>
-      <c r="E374" s="2" t="inlineStr">
+      <c r="E378" s="2" t="inlineStr">
         <is>
           <t>TC_E14S03_03</t>
         </is>
       </c>
-      <c r="F374" s="2" t="inlineStr">
+      <c r="F378" s="2" t="inlineStr">
         <is>
           <t>Both views convert the calendar date across Singapore midnight</t>
         </is>
       </c>
-      <c r="G374" s="2" t="inlineStr">
+      <c r="G378" s="2" t="inlineStr">
         <is>
           <t>Planned, not executed. Controlled local audit fixtures for edited event and registration date/time fields are visible to the Organiser and assigned Coordinator under existing rules.</t>
         </is>
       </c>
-      <c r="H374" s="2" t="inlineStr">
+      <c r="H378" s="2" t="inlineStr">
         <is>
           <t>1. Open the existing Activity log as each permitted reader in turn.
 2. Inspect edited startAt, endAt and registrationDates values using the boundary fixtures, including both endpoints in the existing registrationDates string.
@@ -19994,52 +20199,52 @@
 4. Repeat with a non-Singapore browser timezone.</t>
         </is>
       </c>
-      <c r="I374" s="2" t="inlineStr">
+      <c r="I378" s="2" t="inlineStr">
         <is>
           <t>Boundary values: 2026-10-15T15:59:00Z -&gt; 15 October 23:59 Singapore; 2026-10-15T16:00:00Z -&gt; 16 October 00:00 Singapore; 2026-10-15T18:30:00Z -&gt; 16 October 02:30 Singapore. registrationDates new_value: 2026-10-15T15:59:00Z to 2026-10-15T18:30:00Z (the existing writer's opensAt-to-closesAt form).</t>
         </is>
       </c>
-      <c r="J374" s="2" t="inlineStr">
+      <c r="J378" s="2" t="inlineStr">
         <is>
           <t>Both readers see the correct Singapore calendar day and time for each displayed edited value, including rollover at midnight, independently of browser timezone. Existing display structure is retained.</t>
         </is>
       </c>
     </row>
-    <row r="375">
-      <c r="A375" s="2" t="n">
+    <row r="379">
+      <c r="A379" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B375" s="2" t="inlineStr">
+      <c r="B379" s="2" t="inlineStr">
         <is>
           <t>E14-S03</t>
         </is>
       </c>
-      <c r="C375" s="2" t="inlineStr">
+      <c r="C379" s="2" t="inlineStr">
         <is>
           <t>E14-S03 - Scenario 3</t>
         </is>
       </c>
-      <c r="D375" s="2" t="inlineStr">
+      <c r="D379" s="2" t="inlineStr">
         <is>
           <t>4 - Negative</t>
         </is>
       </c>
-      <c r="E375" s="2" t="inlineStr">
+      <c r="E379" s="2" t="inlineStr">
         <is>
           <t>TC_E14S03_04</t>
         </is>
       </c>
-      <c r="F375" s="2" t="inlineStr">
+      <c r="F379" s="2" t="inlineStr">
         <is>
           <t>Invalid and missing date/time values retain existing helper and omission behavior</t>
         </is>
       </c>
-      <c r="G375" s="2" t="inlineStr">
+      <c r="G379" s="2" t="inlineStr">
         <is>
           <t>Planned, not executed. A local controlled fixture can supply malformed or absent audit change values without modifying production data; note each view's current absent-value display and the shared formatter contract.</t>
         </is>
       </c>
-      <c r="H375" s="2" t="inlineStr">
+      <c r="H379" s="2" t="inlineStr">
         <is>
           <t>1. Supply an invalid nonempty value for an edited date/time field and inspect both existing views.
 2. Repeat with null and empty old/new values.
@@ -20047,52 +20252,52 @@
 4. Check that each view retains its existing absent-value omission/label-only behavior and does not throw.</t>
         </is>
       </c>
-      <c r="I375" s="2" t="inlineStr">
+      <c r="I379" s="2" t="inlineStr">
         <is>
           <t>Edited startAt values: not-a-date, null and empty string; helper-only missing input: undefined.</t>
         </is>
       </c>
-      <c r="J375" s="2" t="inlineStr">
+      <c r="J379" s="2" t="inlineStr">
         <is>
           <t>The existing formatter returns "Not recorded" for missing/invalid input when invoked. Existing absent-value omission/label-only branches remain intact; no invented date, raw invalid date label, new fallback or rendering exception is introduced.</t>
         </is>
       </c>
     </row>
-    <row r="376">
-      <c r="A376" s="2" t="n">
+    <row r="380">
+      <c r="A380" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B376" s="2" t="inlineStr">
+      <c r="B380" s="2" t="inlineStr">
         <is>
           <t>E14-S03</t>
         </is>
       </c>
-      <c r="C376" s="2" t="inlineStr">
+      <c r="C380" s="2" t="inlineStr">
         <is>
           <t>E14-S03 - Scenario 4</t>
         </is>
       </c>
-      <c r="D376" s="2" t="inlineStr">
+      <c r="D380" s="2" t="inlineStr">
         <is>
           <t>3 - Cross-cutting (regression)</t>
         </is>
       </c>
-      <c r="E376" s="2" t="inlineStr">
+      <c r="E380" s="2" t="inlineStr">
         <is>
           <t>TC_E14S03_05</t>
         </is>
       </c>
-      <c r="F376" s="2" t="inlineStr">
+      <c r="F380" s="2" t="inlineStr">
         <is>
           <t>Text, status badges and venue hold expiry are preserved</t>
         </is>
       </c>
-      <c r="G376" s="2" t="inlineStr">
+      <c r="G380" s="2" t="inlineStr">
         <is>
           <t>Planned, not executed. A disposable event has ordinary-text, status-change and venue_booking entries; capture existing expected display behavior for both permitted readers.</t>
         </is>
       </c>
-      <c r="H376" s="2" t="inlineStr">
+      <c r="H380" s="2" t="inlineStr">
         <is>
           <t>1. Open both existing Activity log views and inspect the ordinary-text entry.
 2. Inspect status transitions, including the Coordinator's existing StatusPill badges.
@@ -20100,52 +20305,52 @@
 4. Compare with the existing text/status/hold behavior, keeping unrelated labels and notification text outside the change.</t>
         </is>
       </c>
-      <c r="I376" s="2" t="inlineStr">
+      <c r="I380" s="2" t="inlineStr">
         <is>
           <t>Text title value: 2026-10-15T09:30:00Z (literal title text, not a date field); status: under_review -&gt; approved; venue_booking expiry: 2026-10-15T09:30:00Z; separate booking-id-only entry.</t>
         </is>
       </c>
-      <c r="J376" s="2" t="inlineStr">
+      <c r="J380" s="2" t="inlineStr">
         <is>
           <t>Literal title text is not converted merely because it resembles a timestamp. Status labels and existing badges are unchanged. Existing hold-expiry formatting and booking-id handling remain unchanged; no unrelated action/field-label or notification cleanup is included.</t>
         </is>
       </c>
     </row>
-    <row r="377">
-      <c r="A377" s="2" t="n">
+    <row r="381">
+      <c r="A381" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B377" s="2" t="inlineStr">
+      <c r="B381" s="2" t="inlineStr">
         <is>
           <t>E14-S03</t>
         </is>
       </c>
-      <c r="C377" s="2" t="inlineStr">
+      <c r="C381" s="2" t="inlineStr">
         <is>
           <t>E14-S03 - Scenario 5</t>
         </is>
       </c>
-      <c r="D377" s="2" t="inlineStr">
+      <c r="D381" s="2" t="inlineStr">
         <is>
           <t>3 - Cross-cutting (data isolation)</t>
         </is>
       </c>
-      <c r="E377" s="2" t="inlineStr">
+      <c r="E381" s="2" t="inlineStr">
         <is>
           <t>TC_E14S03_06</t>
         </is>
       </c>
-      <c r="F377" s="2" t="inlineStr">
+      <c r="F381" s="2" t="inlineStr">
         <is>
           <t>Formatting preserves immutable UTC evidence and existing reader access</t>
         </is>
       </c>
-      <c r="G377" s="2" t="inlineStr">
+      <c r="G381" s="2" t="inlineStr">
         <is>
           <t>Planned, not executed. A disposable local database contains an event for one client, its assigned Coordinator, a different-client Organiser, an unassigned Coordinator and an existing access-denial row. A controlled tester snapshots its audit rows read-only.</t>
         </is>
       </c>
-      <c r="H377" s="2" t="inlineStr">
+      <c r="H381" s="2" t="inlineStr">
         <is>
           <t>1. Snapshot old_value, new_value, occurred_at, actor and action for the edited date/time row.
 2. As the permitted Organiser and assigned Coordinator, view and reload the existing log.
@@ -20154,156 +20359,156 @@
 5. Verify event logs still exclude access-denial entries; use the existing TC_E14S02_05 controlled mutation checks for immutability regression.</t>
         </is>
       </c>
-      <c r="I377" s="2" t="inlineStr">
+      <c r="I381" s="2" t="inlineStr">
         <is>
           <t>Stored UTC new_value: 2026-10-15T09:30:00Z; unchanged old_value and occurred_at; unrelated client and unassigned Coordinator; immutable audit row.</t>
         </is>
       </c>
-      <c r="J377" s="2" t="inlineStr">
+      <c r="J381" s="2" t="inlineStr">
         <is>
           <t>Permitted reads format only the presentation: the original stored UTC values, occurrence time, actor and action are unchanged. Existing mutation refusals remain in force, unauthorised readers remain refused without event data, and denial entries stay hidden. No new viewer, permissions or history feature is introduced.</t>
         </is>
       </c>
     </row>
-    <row r="378">
-      <c r="A378" s="2" t="n">
+    <row r="382">
+      <c r="A382" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B378" s="2" t="inlineStr"/>
-      <c r="C378" s="2" t="inlineStr">
+      <c r="B382" s="2" t="inlineStr"/>
+      <c r="C382" s="2" t="inlineStr">
         <is>
           <t>Definition of Done · BDR T-51 · Week 1 §8a</t>
         </is>
       </c>
-      <c r="D378" s="2" t="inlineStr">
+      <c r="D382" s="2" t="inlineStr">
         <is>
           <t>3 - Cross-cutting</t>
         </is>
       </c>
-      <c r="E378" s="2" t="inlineStr">
+      <c r="E382" s="2" t="inlineStr">
         <is>
           <t>TC_PERF_01</t>
         </is>
       </c>
-      <c r="F378" s="2" t="inlineStr">
+      <c r="F382" s="2" t="inlineStr">
         <is>
           <t>Verify a venue search returns within the 3-second target on a realistic catalogue</t>
         </is>
       </c>
-      <c r="G378" s="2" t="inlineStr">
+      <c r="G382" s="2" t="inlineStr">
         <is>
           <t>The venue catalogue holds 50 venues with layouts, accessibility features and facilities. 200 confirmed bookings exist across the next 90 days. Coordinator coord_a@connectsphere.com is signed in</t>
         </is>
       </c>
-      <c r="H378" s="2" t="inlineStr">
+      <c r="H382" s="2" t="inlineStr">
         <is>
           <t>1. Open the venue search
  2. Enter date 2026-12-01, time 09:00–11:00, expected attendance 120, layout Theatre, accessibility Step-free access
  3. Start a timer on submit and stop it when results render</t>
         </is>
       </c>
-      <c r="I378" s="2" t="inlineStr">
+      <c r="I382" s="2" t="inlineStr">
         <is>
           <t>50 venues · 200 bookings · elapsed time measured client-side</t>
         </is>
       </c>
-      <c r="J378" s="2" t="inlineStr">
+      <c r="J382" s="2" t="inlineStr">
         <is>
           <t>Results render in under 3 seconds. Record the measured time; if it exceeds 3 seconds the story does not meet the Definition of Done</t>
         </is>
       </c>
     </row>
-    <row r="379">
-      <c r="A379" s="2" t="n">
+    <row r="383">
+      <c r="A383" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="B379" s="2" t="inlineStr"/>
-      <c r="C379" s="2" t="inlineStr">
+      <c r="B383" s="2" t="inlineStr"/>
+      <c r="C383" s="2" t="inlineStr">
         <is>
           <t>Definition of Done · BDR T-51 · Week 1 §8a</t>
         </is>
       </c>
-      <c r="D379" s="2" t="inlineStr">
+      <c r="D383" s="2" t="inlineStr">
         <is>
           <t>3 - Cross-cutting</t>
         </is>
       </c>
-      <c r="E379" s="2" t="inlineStr">
+      <c r="E383" s="2" t="inlineStr">
         <is>
           <t>TC_PERF_02</t>
         </is>
       </c>
-      <c r="F379" s="2" t="inlineStr">
+      <c r="F383" s="2" t="inlineStr">
         <is>
           <t>Verify the venue availability calendar loads within the 3-second target for a busy month</t>
         </is>
       </c>
-      <c r="G379" s="2" t="inlineStr">
+      <c r="G383" s="2" t="inlineStr">
         <is>
           <t>Orchid Hall has 40 confirmed bookings, 5 tentative holds and 3 maintenance blocks within 2026-12-01 to 2026-12-31</t>
         </is>
       </c>
-      <c r="H379" s="2" t="inlineStr">
+      <c r="H383" s="2" t="inlineStr">
         <is>
           <t>1. Open Orchid Hall in the venue catalogue
  2. Select the calendar for December 2026
  3. Start a timer on selection and stop it when all states have rendered</t>
         </is>
       </c>
-      <c r="I379" s="2" t="inlineStr">
+      <c r="I383" s="2" t="inlineStr">
         <is>
           <t>48 calendar entries in one month · elapsed time measured client-side</t>
         </is>
       </c>
-      <c r="J379" s="2" t="inlineStr">
+      <c r="J383" s="2" t="inlineStr">
         <is>
           <t>The calendar renders all Free, Tentative, Confirmed and Blocked states in under 3 seconds</t>
         </is>
       </c>
     </row>
-    <row r="380">
-      <c r="A380" s="2" t="n">
+    <row r="384">
+      <c r="A384" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="B380" s="2" t="inlineStr"/>
-      <c r="C380" s="2" t="inlineStr">
+      <c r="B384" s="2" t="inlineStr"/>
+      <c r="C384" s="2" t="inlineStr">
         <is>
           <t>Definition of Done · BDR T-51 · Week 1 §8a</t>
         </is>
       </c>
-      <c r="D380" s="2" t="inlineStr">
+      <c r="D384" s="2" t="inlineStr">
         <is>
           <t>3 - Cross-cutting</t>
         </is>
       </c>
-      <c r="E380" s="2" t="inlineStr">
+      <c r="E384" s="2" t="inlineStr">
         <is>
           <t>TC_PERF_03</t>
         </is>
       </c>
-      <c r="F380" s="2" t="inlineStr">
+      <c r="F384" s="2" t="inlineStr">
         <is>
           <t>Verify a registration submission completes within the 3-second target near capacity</t>
         </is>
       </c>
-      <c r="G380" s="2" t="inlineStr">
+      <c r="G384" s="2" t="inlineStr">
         <is>
           <t>Event EVT-2001 is Confirmed with Orchid Hall booked, venue capacity 200, and 198 registrations recorded. Attendee attendee_b@example.com is signed in</t>
         </is>
       </c>
-      <c r="H380" s="2" t="inlineStr">
+      <c r="H384" s="2" t="inlineStr">
         <is>
           <t>1. Open event EVT-2001
  2. Submit a registration
  3. Start a timer on submit and stop it when confirmation renders</t>
         </is>
       </c>
-      <c r="I380" s="2" t="inlineStr">
+      <c r="I384" s="2" t="inlineStr">
         <is>
           <t>198 existing registrations · capacity 200 · elapsed time measured client-side</t>
         </is>
       </c>
-      <c r="J380" s="2" t="inlineStr">
+      <c r="J384" s="2" t="inlineStr">
         <is>
           <t>The registration is created and confirmation renders in under 3 seconds, including the capacity check against the booked venue</t>
         </is>

</xml_diff>

<commit_message>
fix(backend): replan affected requests during Safety Review
Implement the PO-approved E10-S01 interpretation recorded in SCRUM-70 comment 10401. Preserve arrangements and reuse automatic readiness re-entry with fresh SO notification. Parent acceptance remains open.
</commit_message>
<xml_diff>
--- a/docs/testing/PROJECT TEST CASES CAA 311026.xlsx
+++ b/docs/testing/PROJECT TEST CASES CAA 311026.xlsx
@@ -17351,7 +17351,18 @@
       </c>
       <c r="J323" s="2" t="inlineStr">
         <is>
-          <t>"Community Meetup"'s Expected Attendance is updated to 10, and organiser_a@clienta.com is notified that the change was applied</t>
+          <t>"Community Meetup"'s Expected Attendance is updated to 10, and organiser_a@clienta.com is notified that the change was applied
+Safety Review variant (T-103): repeat with an Event in Safety Review and a
+change that flags two Confirmed bookings. Preview leaves the status unchanged;
+applying returns the same Event to Planning and retains both bookings with
+reconfirmation flags. Reconfirming only the first booking leaves it in Planning
+and sends no new SO review request. Reconfirming the last required arrangement
+automatically re-enters Safety Review and sends a fresh SO notification. Repeat
+for an Event in its first Safety Review with no Confirmed history. Preserve
+previous safety decisions without reusing them; require a fresh SO decision.
+Safe-only and structured no-impact changes retain Safety Review. A failed final
+application notice rolls back the Event changes, request status, arrangement
+flags, lifecycle transition, audit and notices together.</t>
         </is>
       </c>
     </row>

</xml_diff>